<commit_message>
Deployed 5550880 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/Buch Bayrische Nächte/Sprache der Hölle.xlsx
+++ b/Buch Bayrische Nächte/Sprache der Hölle.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian Dauner\Documents\GitHub\pnpWiki\docs\Buch Bayrische Nächte\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD4F376F-FFD5-4C39-916C-B98CE95F47AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDBF6526-C138-4A19-B835-3F6C90112E2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="199">
   <si>
     <t>Höllisch</t>
   </si>
@@ -285,9 +285,6 @@
     <t>Pronomen:</t>
   </si>
   <si>
-    <t xml:space="preserve">    Ich:    Ikk</t>
-  </si>
-  <si>
     <t xml:space="preserve">    Du:     Rof</t>
   </si>
   <si>
@@ -333,9 +330,6 @@
     <t xml:space="preserve">        -Osh (Mehrzahl)</t>
   </si>
   <si>
-    <t xml:space="preserve">    Er:     Ash</t>
-  </si>
-  <si>
     <t xml:space="preserve">    Sie (männlich): Shash</t>
   </si>
   <si>
@@ -519,9 +513,6 @@
     <t>Kir-Tra</t>
   </si>
   <si>
-    <t>Ash-Tra</t>
-  </si>
-  <si>
     <t>Mi-Ru-Esch</t>
   </si>
   <si>
@@ -604,6 +595,33 @@
   </si>
   <si>
     <t>Die Sprache der Hölle wird auf die Haut von Höllenbrut geschrieben mit Strähnen aus einem Metall asu der Hölle, welches es nur dort gibt.</t>
+  </si>
+  <si>
+    <t>Ashen-One</t>
+  </si>
+  <si>
+    <t>Born from Ash</t>
+  </si>
+  <si>
+    <t>Born</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Ich:   Ash</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Er:     Ikk</t>
+  </si>
+  <si>
+    <t>Ikk-Tra</t>
+  </si>
+  <si>
+    <t>Born from Ground</t>
+  </si>
+  <si>
+    <t>Ke-Tra</t>
+  </si>
+  <si>
+    <t>Ke-Tra-Ash</t>
   </si>
 </sst>
 </file>
@@ -1127,20 +1145,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AA64"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1" t="s">
         <v>96</v>
-      </c>
-      <c r="B1" t="s">
-        <v>97</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -1164,12 +1182,12 @@
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C2" t="s">
         <v>35</v>
@@ -1214,7 +1232,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -1222,7 +1240,7 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E3" s="6"/>
       <c r="F3" s="7"/>
@@ -1238,15 +1256,15 @@
       <c r="P3" s="7"/>
       <c r="Q3" s="8"/>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>45</v>
       </c>
       <c r="B4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C4" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>53</v>
@@ -1288,15 +1306,15 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>93</v>
+      </c>
+      <c r="B5" t="s">
         <v>94</v>
       </c>
-      <c r="B5" t="s">
-        <v>95</v>
-      </c>
       <c r="C5" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E5" s="9"/>
       <c r="F5" s="1"/>
@@ -1312,15 +1330,15 @@
       <c r="P5" s="1"/>
       <c r="Q5" s="10"/>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C6" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>24</v>
@@ -1392,15 +1410,15 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" t="s">
         <v>105</v>
       </c>
-      <c r="B7" t="s">
-        <v>107</v>
-      </c>
       <c r="C7" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="E7" s="6"/>
       <c r="F7" s="7"/>
@@ -1426,50 +1444,50 @@
       <c r="Z7" s="7"/>
       <c r="AA7" s="8"/>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>104</v>
+      </c>
+      <c r="B8" t="s">
         <v>106</v>
       </c>
-      <c r="B8" t="s">
-        <v>108</v>
-      </c>
       <c r="C8" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="E8" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="F8" s="17" t="s">
+        <v>109</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="I8" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="J8" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="F8" s="17" t="s">
-        <v>111</v>
-      </c>
-      <c r="G8" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="H8" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="I8" s="12" t="s">
+      <c r="K8" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="J8" s="12" t="s">
+      <c r="L8" s="13" t="s">
         <v>116</v>
       </c>
-      <c r="K8" s="12" t="s">
+    </row>
+    <row r="9" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>107</v>
+      </c>
+      <c r="B9" t="s">
         <v>117</v>
       </c>
-      <c r="L8" s="13" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="9" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>109</v>
-      </c>
-      <c r="B9" t="s">
-        <v>119</v>
-      </c>
       <c r="C9" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="E9" s="14">
         <v>0</v>
@@ -1496,191 +1514,191 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B10" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C10" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B11" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C11" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E11" t="s">
         <v>54</v>
       </c>
       <c r="N11" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B12" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C12" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="E12" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B13" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C13" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E13" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B14" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C14" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="E14" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>125</v>
+      </c>
+      <c r="B15" t="s">
+        <v>126</v>
+      </c>
+      <c r="C15" t="s">
+        <v>159</v>
+      </c>
+      <c r="E15" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>127</v>
-      </c>
-      <c r="B15" t="s">
-        <v>128</v>
-      </c>
-      <c r="C15" t="s">
-        <v>161</v>
-      </c>
-      <c r="E15" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
+        <v>141</v>
+      </c>
+      <c r="B16" t="s">
+        <v>142</v>
+      </c>
+      <c r="C16" t="s">
         <v>143</v>
-      </c>
-      <c r="B16" t="s">
-        <v>144</v>
-      </c>
-      <c r="C16" t="s">
-        <v>145</v>
       </c>
       <c r="E16" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B17" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C17" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E17" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B18" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C18" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="E18" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
+        <v>134</v>
+      </c>
+      <c r="B19" t="s">
+        <v>134</v>
+      </c>
+      <c r="C19" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
         <v>136</v>
       </c>
-      <c r="B19" t="s">
-        <v>136</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="B20" t="s">
+        <v>137</v>
+      </c>
+      <c r="C20" t="s">
         <v>135</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>138</v>
-      </c>
-      <c r="B20" t="s">
-        <v>139</v>
-      </c>
-      <c r="C20" t="s">
-        <v>137</v>
       </c>
       <c r="E20" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B21" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C21" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E21" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B22" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C22" t="s">
-        <v>164</v>
+        <v>195</v>
       </c>
       <c r="E22" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B23" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C23" t="s">
         <v>38</v>
@@ -1689,82 +1707,82 @@
         <v>63</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B24" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C24" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="E24" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B25" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C25" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="E25" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
+        <v>164</v>
+      </c>
+      <c r="B26" t="s">
+        <v>165</v>
+      </c>
+      <c r="C26" t="s">
         <v>167</v>
-      </c>
-      <c r="B26" t="s">
-        <v>168</v>
-      </c>
-      <c r="C26" t="s">
-        <v>170</v>
       </c>
       <c r="E26" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B27" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C27" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="E27" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="B28" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="C28" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E28" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B29" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="C29" t="s">
         <v>29</v>
@@ -1773,196 +1791,225 @@
         <v>69</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B30" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="C30" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="E30" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="B31" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C31" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="E31" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B32" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="C32" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="E32" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="B33" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="C33" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="E33" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B34" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="C34" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>192</v>
+      </c>
+      <c r="B35" t="s">
+        <v>196</v>
+      </c>
+      <c r="C35" t="s">
+        <v>197</v>
+      </c>
       <c r="E35" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>48</v>
+      </c>
+      <c r="B36" t="s">
+        <v>48</v>
+      </c>
+      <c r="C36" t="s">
+        <v>48</v>
+      </c>
       <c r="E36" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>190</v>
+      </c>
+      <c r="B37" t="s">
+        <v>191</v>
+      </c>
+      <c r="C37" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E38" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E39" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E41" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E42" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E43" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E44" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E45" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E46" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E48" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="49" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E49" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="50" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E50" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="51" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E51" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="51" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E51" t="s">
+    <row r="52" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E52" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="53" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E53" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="52" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E52" t="s">
+    <row r="54" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E54" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="55" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E55" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="56" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E56" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="57" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E57" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="58" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E58" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="53" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E53" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="54" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E54" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="55" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E55" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="56" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E56" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="57" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E57" t="s">
+    <row r="60" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E60" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="61" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E61" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="58" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E58" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="60" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E60" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="61" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E61" t="s">
+    <row r="62" spans="5:5" x14ac:dyDescent="0.3">
+      <c r="E62" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="62" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E62" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="64" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E64" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deployed 10999ff with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/Buch Bayrische Nächte/Sprache der Hölle.xlsx
+++ b/Buch Bayrische Nächte/Sprache der Hölle.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian Dauner\Documents\GitHub\pnpWiki\docs\Buch Bayrische Nächte\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDBF6526-C138-4A19-B835-3F6C90112E2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00C3CF87-E170-49A6-9EC5-8465AFB8938A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="214">
   <si>
     <t>Höllisch</t>
   </si>
@@ -63,12 +63,6 @@
     <t>Kir</t>
   </si>
   <si>
-    <t>Rfee</t>
-  </si>
-  <si>
-    <t>Krikr</t>
-  </si>
-  <si>
     <t>Tra</t>
   </si>
   <si>
@@ -81,9 +75,6 @@
     <t>Fey</t>
   </si>
   <si>
-    <t>Krok</t>
-  </si>
-  <si>
     <t>Ri</t>
   </si>
   <si>
@@ -96,9 +87,6 @@
     <t>Ikee</t>
   </si>
   <si>
-    <t>Oyf</t>
-  </si>
-  <si>
     <t>Mi</t>
   </si>
   <si>
@@ -117,15 +105,6 @@
     <t>Th</t>
   </si>
   <si>
-    <t>Kv</t>
-  </si>
-  <si>
-    <t>Fr</t>
-  </si>
-  <si>
-    <t>Ht</t>
-  </si>
-  <si>
     <t>To</t>
   </si>
   <si>
@@ -246,9 +225,6 @@
     <t xml:space="preserve">    2+.3. Person plural weiblich</t>
   </si>
   <si>
-    <t xml:space="preserve">        -Krok</t>
-  </si>
-  <si>
     <t xml:space="preserve">    Perfekt:</t>
   </si>
   <si>
@@ -294,24 +270,12 @@
     <t xml:space="preserve">    Wir:    Ikee</t>
   </si>
   <si>
-    <t xml:space="preserve">    Ihr:    Rfee</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Sie (weiblich): Krikr</t>
-  </si>
-  <si>
     <t xml:space="preserve">    Besitzt:        Tra</t>
   </si>
   <si>
-    <t xml:space="preserve">    Wird besitzt:   Oyf</t>
-  </si>
-  <si>
     <t>Death</t>
   </si>
   <si>
-    <t>Death of Souls</t>
-  </si>
-  <si>
     <t>English</t>
   </si>
   <si>
@@ -363,15 +327,6 @@
     <t>Saa</t>
   </si>
   <si>
-    <t>Ko</t>
-  </si>
-  <si>
-    <t>Kt</t>
-  </si>
-  <si>
-    <t>Ksh</t>
-  </si>
-  <si>
     <t>Mo</t>
   </si>
   <si>
@@ -420,9 +375,6 @@
     <t>Other</t>
   </si>
   <si>
-    <t>Pride of Soul</t>
-  </si>
-  <si>
     <t>Ke + Verb</t>
   </si>
   <si>
@@ -480,9 +432,6 @@
     <t>Ley-Tra-Esh</t>
   </si>
   <si>
-    <t>Ru-Hat-Kar</t>
-  </si>
-  <si>
     <t>Ru-Kor</t>
   </si>
   <si>
@@ -492,33 +441,18 @@
     <t>Fuf-Esh</t>
   </si>
   <si>
-    <t>Ru-To-Kor</t>
-  </si>
-  <si>
-    <t>Kir-Ru-To-Kor</t>
-  </si>
-  <si>
     <t>Ke-Osh</t>
   </si>
   <si>
     <t>To-Kar/ To-Esh</t>
   </si>
   <si>
-    <t>Kv-To-Kar</t>
-  </si>
-  <si>
     <t>Ley-To-Esh</t>
   </si>
   <si>
     <t>Kir-Tra</t>
   </si>
   <si>
-    <t>Mi-Ru-Esch</t>
-  </si>
-  <si>
-    <t>Va-Lo-Th-Ay</t>
-  </si>
-  <si>
     <t>tired</t>
   </si>
   <si>
@@ -537,9 +471,6 @@
     <t>Pain of Body</t>
   </si>
   <si>
-    <t>Th-Mi</t>
-  </si>
-  <si>
     <t>Va</t>
   </si>
   <si>
@@ -552,33 +483,15 @@
     <t>and</t>
   </si>
   <si>
-    <t>God of Pain</t>
-  </si>
-  <si>
-    <t>God of Death</t>
-  </si>
-  <si>
-    <t>Body and Soul</t>
-  </si>
-  <si>
     <t>Mi-Esh</t>
   </si>
   <si>
-    <t>Vo-Tra</t>
-  </si>
-  <si>
     <t>Ay-Kar</t>
   </si>
   <si>
     <t>Pains of (Body/Soul)</t>
   </si>
   <si>
-    <t>Va-Lo-Kor</t>
-  </si>
-  <si>
-    <t>Destruction</t>
-  </si>
-  <si>
     <t>Substratction of Time</t>
   </si>
   <si>
@@ -591,21 +504,9 @@
     <t>Lo-Kar</t>
   </si>
   <si>
-    <t>Destruction and Pain</t>
-  </si>
-  <si>
     <t>Die Sprache der Hölle wird auf die Haut von Höllenbrut geschrieben mit Strähnen aus einem Metall asu der Hölle, welches es nur dort gibt.</t>
   </si>
   <si>
-    <t>Ashen-One</t>
-  </si>
-  <si>
-    <t>Born from Ash</t>
-  </si>
-  <si>
-    <t>Born</t>
-  </si>
-  <si>
     <t xml:space="preserve">    Ich:   Ash</t>
   </si>
   <si>
@@ -615,13 +516,157 @@
     <t>Ikk-Tra</t>
   </si>
   <si>
-    <t>Born from Ground</t>
-  </si>
-  <si>
     <t>Ke-Tra</t>
   </si>
   <si>
     <t>Ke-Tra-Ash</t>
+  </si>
+  <si>
+    <t>Ashbearer</t>
+  </si>
+  <si>
+    <t>Bearer of Ash</t>
+  </si>
+  <si>
+    <t>To bear</t>
+  </si>
+  <si>
+    <t>Bear on Ground</t>
+  </si>
+  <si>
+    <t>Kir-Ish</t>
+  </si>
+  <si>
+    <t>Ket</t>
+  </si>
+  <si>
+    <t>Kash</t>
+  </si>
+  <si>
+    <t>Envy</t>
+  </si>
+  <si>
+    <t>Avarice</t>
+  </si>
+  <si>
+    <t>Fury</t>
+  </si>
+  <si>
+    <t>Fer</t>
+  </si>
+  <si>
+    <t>Kvo</t>
+  </si>
+  <si>
+    <t>Kvo-To-Kar</t>
+  </si>
+  <si>
+    <t>Foy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Wird besitzt:  Foy</t>
+  </si>
+  <si>
+    <t>Tuh</t>
+  </si>
+  <si>
+    <t>Nai</t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
+    <t>God</t>
+  </si>
+  <si>
+    <t>Vo-Taa</t>
+  </si>
+  <si>
+    <t>Command</t>
+  </si>
+  <si>
+    <t>to command</t>
+  </si>
+  <si>
+    <t>Het-Erk</t>
+  </si>
+  <si>
+    <t>Sünden</t>
+  </si>
+  <si>
+    <t>Namen der 8 Seelenbändiger (Anagramme zu Wörtern in Höllisch)</t>
+  </si>
+  <si>
+    <t>Pride in Pain</t>
+  </si>
+  <si>
+    <t>Neglect</t>
+  </si>
+  <si>
+    <t>Sorrow</t>
+  </si>
+  <si>
+    <t>Sorrow in Death</t>
+  </si>
+  <si>
+    <t>Anger in Dread</t>
+  </si>
+  <si>
+    <t>All in Completion</t>
+  </si>
+  <si>
+    <t>Envy in Despair</t>
+  </si>
+  <si>
+    <t>Neglect in Desolation</t>
+  </si>
+  <si>
+    <t>Namen der Götter</t>
+  </si>
+  <si>
+    <t>(kein Anagramm)</t>
+  </si>
+  <si>
+    <t>Avarice in Loss</t>
+  </si>
+  <si>
+    <t>Lust</t>
+  </si>
+  <si>
+    <t>Lust in Hunger</t>
+  </si>
+  <si>
+    <t>Loss</t>
+  </si>
+  <si>
+    <t>Krik</t>
+  </si>
+  <si>
+    <t>Rek</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Sie (weiblich): Krik</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Ihr:    Rek</t>
+  </si>
+  <si>
+    <t xml:space="preserve">        -Krof</t>
+  </si>
+  <si>
+    <t>Krof</t>
+  </si>
+  <si>
+    <t>Evil</t>
+  </si>
+  <si>
+    <t>Tuh-Mi</t>
+  </si>
+  <si>
+    <t>Ish Foy Tuh Mi</t>
+  </si>
+  <si>
+    <t>Mo Foy Lo Kar</t>
   </si>
 </sst>
 </file>
@@ -1147,18 +1192,20 @@
   <dimension ref="A1:AA64"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.21875" customWidth="1"/>
+    <col min="20" max="20" width="12.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="B1" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -1184,16 +1231,16 @@
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>145</v>
+        <v>129</v>
       </c>
       <c r="B2" t="s">
-        <v>146</v>
+        <v>130</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>4</v>
@@ -1205,7 +1252,7 @@
         <v>6</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="J2" s="4" t="s">
         <v>7</v>
@@ -1223,13 +1270,13 @@
         <v>11</v>
       </c>
       <c r="O2" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="Q2" s="5" t="s">
         <v>12</v>
-      </c>
-      <c r="P2" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q2" s="5" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1240,7 +1287,7 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>149</v>
+        <v>133</v>
       </c>
       <c r="E3" s="6"/>
       <c r="F3" s="7"/>
@@ -1258,63 +1305,63 @@
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="B4" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="C4" t="s">
-        <v>150</v>
+        <v>134</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="F4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="I4" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="J4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="K4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="L4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="J4" s="4" t="s">
+      <c r="M4" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="N4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="K4" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="L4" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="M4" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="N4" s="4" t="s">
-        <v>22</v>
-      </c>
       <c r="O4" s="4" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="P4" s="4" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>23</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="B5" t="s">
-        <v>94</v>
+        <v>155</v>
       </c>
       <c r="C5" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="E5" s="9"/>
       <c r="F5" s="1"/>
@@ -1332,93 +1379,93 @@
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="B6" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="C6" t="s">
-        <v>152</v>
+        <v>135</v>
       </c>
       <c r="E6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="I6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="F6" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G6" s="4" t="s">
+      <c r="J6" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="L6" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="M6" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="N6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="O6" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="P6" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="Q6" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="K6" s="4" t="s">
+      <c r="R6" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="L6" s="4" t="s">
+      <c r="S6" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="M6" s="4" t="s">
+      <c r="T6" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="N6" s="4" t="s">
+      <c r="U6" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="O6" s="4" t="s">
+      <c r="V6" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="P6" s="4" t="s">
+      <c r="W6" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="Q6" s="4" t="s">
+      <c r="X6" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y6" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="R6" s="4" t="s">
+      <c r="Z6" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="S6" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="T6" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="U6" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="V6" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="W6" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="X6" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="Y6" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="Z6" s="4" t="s">
-        <v>44</v>
-      </c>
       <c r="AA6" s="5" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="B7" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="C7" t="s">
-        <v>153</v>
+        <v>136</v>
       </c>
       <c r="E7" s="6"/>
       <c r="F7" s="7"/>
@@ -1446,48 +1493,48 @@
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="B8" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="C8" t="s">
-        <v>154</v>
+        <v>137</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>112</v>
+        <v>181</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>110</v>
+        <v>98</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="I8" s="12" t="s">
-        <v>113</v>
+        <v>170</v>
       </c>
       <c r="J8" s="12" t="s">
-        <v>114</v>
+        <v>171</v>
       </c>
       <c r="K8" s="12" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="L8" s="13" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
     </row>
     <row r="9" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="B9" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="C9" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="E9" s="14">
         <v>0</v>
@@ -1516,503 +1563,623 @@
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="B10" t="s">
-        <v>131</v>
+        <v>105</v>
       </c>
       <c r="C10" t="s">
-        <v>155</v>
+        <v>97</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="B11" t="s">
-        <v>119</v>
+        <v>104</v>
       </c>
       <c r="C11" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="E11" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="N11" t="s">
-        <v>189</v>
+        <v>159</v>
       </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="B12" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="C12" t="s">
-        <v>157</v>
+        <v>138</v>
       </c>
       <c r="E12" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>123</v>
+        <v>108</v>
       </c>
       <c r="B13" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="C13" t="s">
-        <v>132</v>
+        <v>116</v>
       </c>
       <c r="E13" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>127</v>
+        <v>112</v>
       </c>
       <c r="B14" t="s">
-        <v>127</v>
+        <v>112</v>
       </c>
       <c r="C14" t="s">
-        <v>158</v>
+        <v>139</v>
       </c>
       <c r="E14" t="s">
-        <v>99</v>
+        <v>87</v>
+      </c>
+      <c r="N14" t="s">
+        <v>188</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>198</v>
+      </c>
+      <c r="T14" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>125</v>
+        <v>110</v>
       </c>
       <c r="B15" t="s">
-        <v>126</v>
+        <v>111</v>
       </c>
       <c r="C15" t="s">
-        <v>159</v>
+        <v>177</v>
       </c>
       <c r="E15" t="s">
-        <v>100</v>
+        <v>88</v>
+      </c>
+      <c r="N15" t="s">
+        <v>182</v>
+      </c>
+      <c r="O15" t="s">
+        <v>181</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>195</v>
+      </c>
+      <c r="U15" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
+        <v>125</v>
+      </c>
+      <c r="B16" t="s">
+        <v>126</v>
+      </c>
+      <c r="C16" t="s">
+        <v>127</v>
+      </c>
+      <c r="E16" t="s">
+        <v>50</v>
+      </c>
+      <c r="N16" t="s">
+        <v>105</v>
+      </c>
+      <c r="O16" t="s">
+        <v>97</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>190</v>
+      </c>
+      <c r="S16" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>115</v>
+      </c>
+      <c r="B17" t="s">
+        <v>115</v>
+      </c>
+      <c r="C17" t="s">
+        <v>133</v>
+      </c>
+      <c r="E17" t="s">
+        <v>51</v>
+      </c>
+      <c r="N17" t="s">
+        <v>201</v>
+      </c>
+      <c r="O17" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>113</v>
+      </c>
+      <c r="B18" t="s">
+        <v>114</v>
+      </c>
+      <c r="C18" t="s">
+        <v>140</v>
+      </c>
+      <c r="E18" t="s">
+        <v>52</v>
+      </c>
+      <c r="N18" t="s">
+        <v>191</v>
+      </c>
+      <c r="O18" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>118</v>
+      </c>
+      <c r="B19" t="s">
+        <v>118</v>
+      </c>
+      <c r="C19" t="s">
+        <v>117</v>
+      </c>
+      <c r="N19" t="s">
+        <v>172</v>
+      </c>
+      <c r="O19" t="s">
+        <v>170</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>120</v>
+      </c>
+      <c r="B20" t="s">
+        <v>121</v>
+      </c>
+      <c r="C20" t="s">
+        <v>119</v>
+      </c>
+      <c r="E20" t="s">
+        <v>53</v>
+      </c>
+      <c r="N20" t="s">
+        <v>173</v>
+      </c>
+      <c r="O20" t="s">
+        <v>171</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>122</v>
+      </c>
+      <c r="B21" t="s">
+        <v>122</v>
+      </c>
+      <c r="C21" t="s">
         <v>141</v>
       </c>
-      <c r="B16" t="s">
+      <c r="E21" t="s">
+        <v>54</v>
+      </c>
+      <c r="N21" t="s">
+        <v>192</v>
+      </c>
+      <c r="O21" t="s">
+        <v>100</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>193</v>
+      </c>
+      <c r="S21" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>123</v>
+      </c>
+      <c r="B22" t="s">
+        <v>123</v>
+      </c>
+      <c r="C22" t="s">
+        <v>162</v>
+      </c>
+      <c r="E22" t="s">
+        <v>55</v>
+      </c>
+      <c r="N22" t="s">
+        <v>174</v>
+      </c>
+      <c r="O22" t="s">
+        <v>101</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>124</v>
+      </c>
+      <c r="B23" t="s">
+        <v>124</v>
+      </c>
+      <c r="C23" t="s">
+        <v>31</v>
+      </c>
+      <c r="E23" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>131</v>
+      </c>
+      <c r="B24" t="s">
+        <v>132</v>
+      </c>
+      <c r="C24" t="s">
+        <v>184</v>
+      </c>
+      <c r="E24" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>144</v>
+      </c>
+      <c r="B25" t="s">
+        <v>144</v>
+      </c>
+      <c r="C25" t="s">
+        <v>152</v>
+      </c>
+      <c r="E25" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
         <v>142</v>
       </c>
-      <c r="C16" t="s">
+      <c r="B26" t="s">
         <v>143</v>
       </c>
-      <c r="E16" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>130</v>
-      </c>
-      <c r="B17" t="s">
-        <v>130</v>
-      </c>
-      <c r="C17" t="s">
+      <c r="C26" t="s">
+        <v>145</v>
+      </c>
+      <c r="E26" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>146</v>
+      </c>
+      <c r="B27" t="s">
+        <v>147</v>
+      </c>
+      <c r="C27" t="s">
+        <v>211</v>
+      </c>
+      <c r="E27" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
         <v>149</v>
       </c>
-      <c r="E17" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>128</v>
-      </c>
-      <c r="B18" t="s">
-        <v>129</v>
-      </c>
-      <c r="C18" t="s">
-        <v>160</v>
-      </c>
-      <c r="E18" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>134</v>
-      </c>
-      <c r="B19" t="s">
-        <v>134</v>
-      </c>
-      <c r="C19" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>136</v>
-      </c>
-      <c r="B20" t="s">
-        <v>137</v>
-      </c>
-      <c r="C20" t="s">
-        <v>135</v>
-      </c>
-      <c r="E20" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>138</v>
-      </c>
-      <c r="B21" t="s">
-        <v>138</v>
-      </c>
-      <c r="C21" t="s">
-        <v>161</v>
-      </c>
-      <c r="E21" t="s">
+      <c r="B28" t="s">
+        <v>150</v>
+      </c>
+      <c r="C28" t="s">
+        <v>148</v>
+      </c>
+      <c r="E28" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>139</v>
-      </c>
-      <c r="B22" t="s">
-        <v>139</v>
-      </c>
-      <c r="C22" t="s">
-        <v>195</v>
-      </c>
-      <c r="E22" t="s">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>151</v>
+      </c>
+      <c r="B29" t="s">
+        <v>151</v>
+      </c>
+      <c r="C29" t="s">
+        <v>25</v>
+      </c>
+      <c r="E29" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>140</v>
-      </c>
-      <c r="B23" t="s">
-        <v>140</v>
-      </c>
-      <c r="C23" t="s">
-        <v>38</v>
-      </c>
-      <c r="E23" t="s">
+    <row r="30" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>156</v>
+      </c>
+      <c r="B30" t="s">
+        <v>157</v>
+      </c>
+      <c r="C30" t="s">
+        <v>22</v>
+      </c>
+      <c r="E30" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>147</v>
-      </c>
-      <c r="B24" t="s">
-        <v>148</v>
-      </c>
-      <c r="C24" t="s">
-        <v>179</v>
-      </c>
-      <c r="E24" t="s">
+    <row r="31" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>203</v>
+      </c>
+      <c r="B31" t="s">
+        <v>203</v>
+      </c>
+      <c r="C31" t="s">
+        <v>13</v>
+      </c>
+      <c r="E31" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>166</v>
-      </c>
-      <c r="B25" t="s">
-        <v>166</v>
-      </c>
-      <c r="C25" t="s">
-        <v>178</v>
-      </c>
-      <c r="E25" t="s">
+    <row r="32" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>82</v>
+      </c>
+      <c r="B32" t="s">
+        <v>155</v>
+      </c>
+      <c r="C32" t="s">
+        <v>158</v>
+      </c>
+      <c r="E32" t="s">
         <v>65</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>164</v>
-      </c>
-      <c r="B26" t="s">
-        <v>165</v>
-      </c>
-      <c r="C26" t="s">
-        <v>167</v>
-      </c>
-      <c r="E26" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>168</v>
-      </c>
-      <c r="B27" t="s">
-        <v>169</v>
-      </c>
-      <c r="C27" t="s">
-        <v>170</v>
-      </c>
-      <c r="E27" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>172</v>
-      </c>
-      <c r="B28" t="s">
-        <v>173</v>
-      </c>
-      <c r="C28" t="s">
-        <v>171</v>
-      </c>
-      <c r="E28" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>174</v>
-      </c>
-      <c r="B29" t="s">
-        <v>174</v>
-      </c>
-      <c r="C29" t="s">
-        <v>29</v>
-      </c>
-      <c r="E29" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>185</v>
-      </c>
-      <c r="B30" t="s">
-        <v>186</v>
-      </c>
-      <c r="C30" t="s">
-        <v>187</v>
-      </c>
-      <c r="E30" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>183</v>
-      </c>
-      <c r="B31" t="s">
-        <v>184</v>
-      </c>
-      <c r="C31" t="s">
-        <v>182</v>
-      </c>
-      <c r="E31" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>168</v>
-      </c>
-      <c r="B32" t="s">
-        <v>181</v>
-      </c>
-      <c r="C32" t="s">
-        <v>180</v>
-      </c>
-      <c r="E32" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>176</v>
+        <v>146</v>
       </c>
       <c r="B33" t="s">
-        <v>177</v>
+        <v>154</v>
       </c>
       <c r="C33" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="E33" t="s">
-        <v>73</v>
+        <v>208</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>175</v>
+        <v>210</v>
       </c>
       <c r="B34" t="s">
-        <v>188</v>
+        <v>210</v>
       </c>
       <c r="C34" t="s">
-        <v>163</v>
+        <v>176</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>192</v>
+        <v>167</v>
       </c>
       <c r="B35" t="s">
-        <v>196</v>
+        <v>168</v>
       </c>
       <c r="C35" t="s">
-        <v>197</v>
+        <v>163</v>
       </c>
       <c r="E35" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="B36" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="C36" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="E36" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>190</v>
+        <v>165</v>
       </c>
       <c r="B37" t="s">
-        <v>191</v>
+        <v>166</v>
       </c>
       <c r="C37" t="s">
-        <v>198</v>
+        <v>164</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>183</v>
+      </c>
+      <c r="B38" t="s">
+        <v>182</v>
+      </c>
+      <c r="C38" t="s">
+        <v>181</v>
+      </c>
       <c r="E38" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>185</v>
+      </c>
+      <c r="B39" t="s">
+        <v>185</v>
+      </c>
+      <c r="C39" t="s">
+        <v>101</v>
+      </c>
       <c r="E39" t="s">
-        <v>77</v>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>186</v>
+      </c>
+      <c r="B40" t="s">
+        <v>186</v>
+      </c>
+      <c r="C40" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E41" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E42" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E43" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E44" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E45" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E46" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E48" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
     </row>
     <row r="49" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E49" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
     </row>
     <row r="50" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E50" t="s">
-        <v>193</v>
+        <v>160</v>
       </c>
     </row>
     <row r="51" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E51" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
     </row>
     <row r="52" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E52" t="s">
-        <v>194</v>
+        <v>161</v>
       </c>
     </row>
     <row r="53" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E53" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
     </row>
     <row r="54" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E54" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
     </row>
     <row r="55" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E55" t="s">
-        <v>89</v>
+        <v>207</v>
       </c>
     </row>
     <row r="56" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E56" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
     </row>
     <row r="57" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E57" t="s">
-        <v>90</v>
+        <v>206</v>
       </c>
     </row>
     <row r="58" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E58" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
     </row>
     <row r="60" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E60" t="s">
-        <v>144</v>
+        <v>128</v>
       </c>
     </row>
     <row r="61" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E61" t="s">
-        <v>91</v>
+        <v>81</v>
       </c>
     </row>
     <row r="62" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E62" t="s">
-        <v>92</v>
+        <v>179</v>
       </c>
     </row>
     <row r="64" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E64" t="s">
-        <v>108</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Deployed eec42b8 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/Buch Bayrische Nächte/Sprache der Hölle.xlsx
+++ b/Buch Bayrische Nächte/Sprache der Hölle.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian Dauner\Documents\GitHub\pnpWiki\docs\Buch Bayrische Nächte\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00C3CF87-E170-49A6-9EC5-8465AFB8938A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64D48BF2-F39B-4274-AFB0-E8AF665ABC44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="265">
   <si>
     <t>Höllisch</t>
   </si>
@@ -81,9 +81,6 @@
     <t>Tat</t>
   </si>
   <si>
-    <t>Ikk</t>
-  </si>
-  <si>
     <t>Ikee</t>
   </si>
   <si>
@@ -102,9 +99,6 @@
     <t>Ru</t>
   </si>
   <si>
-    <t>Th</t>
-  </si>
-  <si>
     <t>To</t>
   </si>
   <si>
@@ -423,9 +417,6 @@
     <t>humanlike</t>
   </si>
   <si>
-    <t>naked, industrious</t>
-  </si>
-  <si>
     <t>Ley-Esh</t>
   </si>
   <si>
@@ -441,9 +432,6 @@
     <t>Fuf-Esh</t>
   </si>
   <si>
-    <t>Ke-Osh</t>
-  </si>
-  <si>
     <t>To-Kar/ To-Esh</t>
   </si>
   <si>
@@ -477,9 +465,6 @@
     <t>less</t>
   </si>
   <si>
-    <t>substraction from</t>
-  </si>
-  <si>
     <t>and</t>
   </si>
   <si>
@@ -531,9 +516,6 @@
     <t>To bear</t>
   </si>
   <si>
-    <t>Bear on Ground</t>
-  </si>
-  <si>
     <t>Kir-Ish</t>
   </si>
   <si>
@@ -597,27 +579,15 @@
     <t>Namen der 8 Seelenbändiger (Anagramme zu Wörtern in Höllisch)</t>
   </si>
   <si>
-    <t>Pride in Pain</t>
-  </si>
-  <si>
     <t>Neglect</t>
   </si>
   <si>
     <t>Sorrow</t>
   </si>
   <si>
-    <t>Sorrow in Death</t>
-  </si>
-  <si>
-    <t>Anger in Dread</t>
-  </si>
-  <si>
     <t>All in Completion</t>
   </si>
   <si>
-    <t>Envy in Despair</t>
-  </si>
-  <si>
     <t>Neglect in Desolation</t>
   </si>
   <si>
@@ -663,10 +633,193 @@
     <t>Tuh-Mi</t>
   </si>
   <si>
-    <t>Ish Foy Tuh Mi</t>
-  </si>
-  <si>
-    <t>Mo Foy Lo Kar</t>
+    <t>Completion</t>
+  </si>
+  <si>
+    <t>Ish-Foy-Tuh-Mi</t>
+  </si>
+  <si>
+    <t>Mo-Foy-Lo-Kar</t>
+  </si>
+  <si>
+    <t>Abkürzung</t>
+  </si>
+  <si>
+    <t>Für Namen werden die Wörter in ein neues Wort abgekürzt, unabhängig vom Alphabet. Geschrieben werden sie direkt zusammen, ohne Silbentrennung.</t>
+  </si>
+  <si>
+    <t>Mofylkar</t>
+  </si>
+  <si>
+    <t>Completion of All</t>
+  </si>
+  <si>
+    <t>Oor-Nai</t>
+  </si>
+  <si>
+    <t>Nai-Tra-Oor-Nai</t>
+  </si>
+  <si>
+    <t>Naitronai</t>
+  </si>
+  <si>
+    <t>Pride out of Pain</t>
+  </si>
+  <si>
+    <t>Envy out of Despair</t>
+  </si>
+  <si>
+    <t>Sorrow out of Death</t>
+  </si>
+  <si>
+    <t>Anger out of Dread</t>
+  </si>
+  <si>
+    <t>Hunger</t>
+  </si>
+  <si>
+    <t>Fullness</t>
+  </si>
+  <si>
+    <t>Absence of Fullness</t>
+  </si>
+  <si>
+    <t>Va-Raa</t>
+  </si>
+  <si>
+    <t>substraction from/absence</t>
+  </si>
+  <si>
+    <t>Nir-Tra-Va-Raa</t>
+  </si>
+  <si>
+    <t>Nirtravra</t>
+  </si>
+  <si>
+    <t>Desolation</t>
+  </si>
+  <si>
+    <t>Fire</t>
+  </si>
+  <si>
+    <t>Ikt</t>
+  </si>
+  <si>
+    <t>Fire on Ground</t>
+  </si>
+  <si>
+    <t>to bear on Ground</t>
+  </si>
+  <si>
+    <t>Ri-Ke</t>
+  </si>
+  <si>
+    <t>Saa-Tra-Ri-Ke</t>
+  </si>
+  <si>
+    <t>Ishfotum</t>
+  </si>
+  <si>
+    <t>Sadness</t>
+  </si>
+  <si>
+    <t>Despair</t>
+  </si>
+  <si>
+    <t>greatest Sadness</t>
+  </si>
+  <si>
+    <t>Fer-Ref</t>
+  </si>
+  <si>
+    <t>Ket-Foy-Fer-Ref</t>
+  </si>
+  <si>
+    <t>Ketfyref</t>
+  </si>
+  <si>
+    <t>Less</t>
+  </si>
+  <si>
+    <t>Veek-Kar</t>
+  </si>
+  <si>
+    <t>more of Less</t>
+  </si>
+  <si>
+    <t>Kash-Tra-Veek-Kar</t>
+  </si>
+  <si>
+    <t>Kashtravkar</t>
+  </si>
+  <si>
+    <t>Fear</t>
+  </si>
+  <si>
+    <t>Dread</t>
+  </si>
+  <si>
+    <t>More of Fear</t>
+  </si>
+  <si>
+    <t>Shi-Kar</t>
+  </si>
+  <si>
+    <t>Het-Foy-Shi-Kar</t>
+  </si>
+  <si>
+    <t>Hetfoshkar</t>
+  </si>
+  <si>
+    <t>Saatrark</t>
+  </si>
+  <si>
+    <t>Irnatrav'Ara</t>
+  </si>
+  <si>
+    <t>Asarat'Rike</t>
+  </si>
+  <si>
+    <t>Shkaratve'Kekar</t>
+  </si>
+  <si>
+    <t>Ethfyosh'Ikar</t>
+  </si>
+  <si>
+    <t>Naitro'Nai</t>
+  </si>
+  <si>
+    <t>Shiofthu'Mi</t>
+  </si>
+  <si>
+    <t>Omofy'Olrak</t>
+  </si>
+  <si>
+    <t>Tekofy'Erffar</t>
+  </si>
+  <si>
+    <t>Belonging</t>
+  </si>
+  <si>
+    <t>from</t>
+  </si>
+  <si>
+    <t>Ke-Kar</t>
+  </si>
+  <si>
+    <t>Strength</t>
+  </si>
+  <si>
+    <t>Earthly strength</t>
+  </si>
+  <si>
+    <t>Ke-Kar-Vo-Ash</t>
+  </si>
+  <si>
+    <t>Strength of Ash</t>
+  </si>
+  <si>
+    <t>Strength of Ashbearers</t>
   </si>
 </sst>
 </file>
@@ -1193,19 +1346,21 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="13.21875" customWidth="1"/>
+    <col min="18" max="18" width="11.21875" customWidth="1"/>
+    <col min="19" max="19" width="17" customWidth="1"/>
     <col min="20" max="20" width="12.33203125" customWidth="1"/>
+    <col min="22" max="22" width="13.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -1231,16 +1386,16 @@
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>4</v>
@@ -1252,7 +1407,7 @@
         <v>6</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="J2" s="4" t="s">
         <v>7</v>
@@ -1270,10 +1425,10 @@
         <v>11</v>
       </c>
       <c r="O2" s="4" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="P2" s="4" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="Q2" s="5" t="s">
         <v>12</v>
@@ -1287,7 +1442,7 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="E3" s="6"/>
       <c r="F3" s="7"/>
@@ -1305,16 +1460,16 @@
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C4" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>13</v>
@@ -1326,7 +1481,7 @@
         <v>15</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="J4" s="4" t="s">
         <v>16</v>
@@ -1335,34 +1490,25 @@
         <v>17</v>
       </c>
       <c r="L4" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="M4" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="N4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="M4" s="4" t="s">
+      <c r="O4" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="P4" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="N4" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="O4" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="P4" s="4" t="s">
-        <v>43</v>
-      </c>
       <c r="Q4" s="5" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
     </row>
     <row r="5" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>82</v>
-      </c>
-      <c r="B5" t="s">
-        <v>155</v>
-      </c>
-      <c r="C5" t="s">
-        <v>158</v>
-      </c>
       <c r="E5" s="9"/>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
@@ -1379,93 +1525,93 @@
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B6" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C6" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="E6" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="G6" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="H6" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="I6" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="J6" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="K6" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="L6" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="M6" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="N6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="J6" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="L6" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="M6" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="N6" s="4" t="s">
+      <c r="O6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="P6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="O6" s="4" t="s">
+      <c r="Q6" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="P6" s="4" t="s">
+      <c r="R6" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="Q6" s="4" t="s">
+      <c r="S6" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="R6" s="4" t="s">
+      <c r="T6" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="S6" s="4" t="s">
+      <c r="U6" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="T6" s="4" t="s">
+      <c r="V6" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="U6" s="4" t="s">
+      <c r="W6" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="V6" s="4" t="s">
+      <c r="X6" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y6" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="W6" s="4" t="s">
+      <c r="Z6" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="X6" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="Y6" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="Z6" s="4" t="s">
-        <v>37</v>
-      </c>
       <c r="AA6" s="5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B7" t="s">
         <v>91</v>
       </c>
-      <c r="B7" t="s">
-        <v>93</v>
-      </c>
       <c r="C7" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="E7" s="6"/>
       <c r="F7" s="7"/>
@@ -1493,48 +1639,48 @@
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>90</v>
+      </c>
+      <c r="B8" t="s">
         <v>92</v>
       </c>
-      <c r="B8" t="s">
-        <v>94</v>
-      </c>
       <c r="C8" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="F8" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="H8" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="G8" s="12" t="s">
+      <c r="I8" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="J8" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="K8" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="H8" s="12" t="s">
+      <c r="L8" s="13" t="s">
         <v>99</v>
-      </c>
-      <c r="I8" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="J8" s="12" t="s">
-        <v>171</v>
-      </c>
-      <c r="K8" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="L8" s="13" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="9" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B9" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C9" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="E9" s="14">
         <v>0</v>
@@ -1563,619 +1709,813 @@
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C10" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B11" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C11" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="E11" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="N11" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B12" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C12" t="s">
-        <v>138</v>
+        <v>22</v>
       </c>
       <c r="E12" t="s">
-        <v>48</v>
+        <v>46</v>
+      </c>
+      <c r="N12" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B13" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C13" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E13" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B14" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C14" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="E14" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="N14" t="s">
+        <v>182</v>
+      </c>
+      <c r="Q14" t="s">
         <v>188</v>
       </c>
-      <c r="Q14" t="s">
-        <v>198</v>
+      <c r="S14" t="s">
+        <v>0</v>
       </c>
       <c r="T14" t="s">
-        <v>189</v>
+        <v>205</v>
+      </c>
+      <c r="V14" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B15" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C15" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="E15" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="N15" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="O15" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="Q15" t="s">
-        <v>195</v>
-      </c>
-      <c r="U15" t="s">
-        <v>199</v>
+        <v>186</v>
+      </c>
+      <c r="S15" t="s">
+        <v>210</v>
+      </c>
+      <c r="T15" t="s">
+        <v>211</v>
+      </c>
+      <c r="V15" t="s">
+        <v>253</v>
+      </c>
+      <c r="W15" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
+        <v>123</v>
+      </c>
+      <c r="B16" t="s">
+        <v>124</v>
+      </c>
+      <c r="C16" t="s">
         <v>125</v>
       </c>
-      <c r="B16" t="s">
-        <v>126</v>
-      </c>
-      <c r="C16" t="s">
-        <v>127</v>
-      </c>
       <c r="E16" t="s">
+        <v>48</v>
+      </c>
+      <c r="N16" t="s">
+        <v>103</v>
+      </c>
+      <c r="O16" t="s">
+        <v>95</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>212</v>
+      </c>
+      <c r="S16" t="s">
+        <v>203</v>
+      </c>
+      <c r="T16" t="s">
+        <v>230</v>
+      </c>
+      <c r="V16" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="17" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>113</v>
+      </c>
+      <c r="B17" t="s">
+        <v>113</v>
+      </c>
+      <c r="C17" t="s">
+        <v>130</v>
+      </c>
+      <c r="E17" t="s">
+        <v>49</v>
+      </c>
+      <c r="N17" t="s">
+        <v>191</v>
+      </c>
+      <c r="O17" t="s">
+        <v>96</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>192</v>
+      </c>
+      <c r="S17" t="s">
+        <v>221</v>
+      </c>
+      <c r="T17" t="s">
+        <v>222</v>
+      </c>
+      <c r="V17" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>111</v>
+      </c>
+      <c r="B18" t="s">
+        <v>112</v>
+      </c>
+      <c r="C18" t="s">
+        <v>136</v>
+      </c>
+      <c r="E18" t="s">
         <v>50</v>
       </c>
-      <c r="N16" t="s">
-        <v>105</v>
-      </c>
-      <c r="O16" t="s">
+      <c r="N18" t="s">
+        <v>184</v>
+      </c>
+      <c r="O18" t="s">
         <v>97</v>
       </c>
-      <c r="Q16" t="s">
+      <c r="Q18" t="s">
+        <v>187</v>
+      </c>
+      <c r="S18" t="s">
+        <v>229</v>
+      </c>
+      <c r="T18" t="s">
+        <v>248</v>
+      </c>
+      <c r="V18" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="19" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>116</v>
+      </c>
+      <c r="B19" t="s">
+        <v>116</v>
+      </c>
+      <c r="C19" t="s">
+        <v>115</v>
+      </c>
+      <c r="N19" t="s">
+        <v>166</v>
+      </c>
+      <c r="O19" t="s">
+        <v>164</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>213</v>
+      </c>
+      <c r="S19" t="s">
+        <v>235</v>
+      </c>
+      <c r="T19" t="s">
+        <v>236</v>
+      </c>
+      <c r="V19" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="20" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>118</v>
+      </c>
+      <c r="B20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C20" t="s">
+        <v>117</v>
+      </c>
+      <c r="E20" t="s">
+        <v>51</v>
+      </c>
+      <c r="N20" t="s">
+        <v>167</v>
+      </c>
+      <c r="O20" t="s">
+        <v>165</v>
+      </c>
+      <c r="Q20" t="s">
         <v>190</v>
       </c>
-      <c r="S16" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>115</v>
-      </c>
-      <c r="B17" t="s">
-        <v>115</v>
-      </c>
-      <c r="C17" t="s">
-        <v>133</v>
-      </c>
-      <c r="E17" t="s">
-        <v>51</v>
-      </c>
-      <c r="N17" t="s">
+      <c r="S20" t="s">
+        <v>240</v>
+      </c>
+      <c r="T20" t="s">
+        <v>241</v>
+      </c>
+      <c r="V20" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="21" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>120</v>
+      </c>
+      <c r="B21" t="s">
+        <v>120</v>
+      </c>
+      <c r="C21" t="s">
+        <v>137</v>
+      </c>
+      <c r="E21" t="s">
+        <v>52</v>
+      </c>
+      <c r="N21" t="s">
+        <v>185</v>
+      </c>
+      <c r="O21" t="s">
+        <v>98</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>214</v>
+      </c>
+      <c r="S21" t="s">
+        <v>204</v>
+      </c>
+      <c r="T21" t="s">
+        <v>207</v>
+      </c>
+      <c r="V21" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="22" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>121</v>
+      </c>
+      <c r="B22" t="s">
+        <v>121</v>
+      </c>
+      <c r="C22" t="s">
+        <v>157</v>
+      </c>
+      <c r="E22" t="s">
+        <v>53</v>
+      </c>
+      <c r="N22" t="s">
+        <v>168</v>
+      </c>
+      <c r="O22" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>215</v>
+      </c>
+      <c r="S22" t="s">
+        <v>246</v>
+      </c>
+      <c r="T22" t="s">
+        <v>247</v>
+      </c>
+      <c r="V22" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="23" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>122</v>
+      </c>
+      <c r="B23" t="s">
+        <v>122</v>
+      </c>
+      <c r="C23" t="s">
+        <v>29</v>
+      </c>
+      <c r="E23" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="24" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>129</v>
+      </c>
+      <c r="B24" t="s">
+        <v>257</v>
+      </c>
+      <c r="C24" t="s">
+        <v>178</v>
+      </c>
+      <c r="E24" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="25" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>140</v>
+      </c>
+      <c r="B25" t="s">
+        <v>140</v>
+      </c>
+      <c r="C25" t="s">
+        <v>147</v>
+      </c>
+      <c r="E25" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="26" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>138</v>
+      </c>
+      <c r="B26" t="s">
+        <v>139</v>
+      </c>
+      <c r="C26" t="s">
+        <v>141</v>
+      </c>
+      <c r="E26" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="27" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>142</v>
+      </c>
+      <c r="B27" t="s">
+        <v>143</v>
+      </c>
+      <c r="C27" t="s">
         <v>201</v>
       </c>
-      <c r="O17" t="s">
-        <v>98</v>
-      </c>
-      <c r="Q17" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>113</v>
-      </c>
-      <c r="B18" t="s">
-        <v>114</v>
-      </c>
-      <c r="C18" t="s">
-        <v>140</v>
-      </c>
-      <c r="E18" t="s">
-        <v>52</v>
-      </c>
-      <c r="N18" t="s">
-        <v>191</v>
-      </c>
-      <c r="O18" t="s">
-        <v>99</v>
-      </c>
-      <c r="Q18" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>118</v>
-      </c>
-      <c r="B19" t="s">
-        <v>118</v>
-      </c>
-      <c r="C19" t="s">
-        <v>117</v>
-      </c>
-      <c r="N19" t="s">
-        <v>172</v>
-      </c>
-      <c r="O19" t="s">
-        <v>170</v>
-      </c>
-      <c r="Q19" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>120</v>
-      </c>
-      <c r="B20" t="s">
-        <v>121</v>
-      </c>
-      <c r="C20" t="s">
-        <v>119</v>
-      </c>
-      <c r="E20" t="s">
-        <v>53</v>
-      </c>
-      <c r="N20" t="s">
-        <v>173</v>
-      </c>
-      <c r="O20" t="s">
-        <v>171</v>
-      </c>
-      <c r="Q20" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>122</v>
-      </c>
-      <c r="B21" t="s">
-        <v>122</v>
-      </c>
-      <c r="C21" t="s">
-        <v>141</v>
-      </c>
-      <c r="E21" t="s">
-        <v>54</v>
-      </c>
-      <c r="N21" t="s">
-        <v>192</v>
-      </c>
-      <c r="O21" t="s">
-        <v>100</v>
-      </c>
-      <c r="Q21" t="s">
-        <v>193</v>
-      </c>
-      <c r="S21" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>123</v>
-      </c>
-      <c r="B22" t="s">
-        <v>123</v>
-      </c>
-      <c r="C22" t="s">
-        <v>162</v>
-      </c>
-      <c r="E22" t="s">
-        <v>55</v>
-      </c>
-      <c r="N22" t="s">
-        <v>174</v>
-      </c>
-      <c r="O22" t="s">
-        <v>101</v>
-      </c>
-      <c r="Q22" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>124</v>
-      </c>
-      <c r="B23" t="s">
-        <v>124</v>
-      </c>
-      <c r="C23" t="s">
-        <v>31</v>
-      </c>
-      <c r="E23" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>131</v>
-      </c>
-      <c r="B24" t="s">
-        <v>132</v>
-      </c>
-      <c r="C24" t="s">
-        <v>184</v>
-      </c>
-      <c r="E24" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+      <c r="E27" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="28" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>145</v>
+      </c>
+      <c r="B28" t="s">
+        <v>220</v>
+      </c>
+      <c r="C28" t="s">
         <v>144</v>
       </c>
-      <c r="B25" t="s">
-        <v>144</v>
-      </c>
-      <c r="C25" t="s">
+      <c r="E28" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="29" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>146</v>
+      </c>
+      <c r="B29" t="s">
+        <v>146</v>
+      </c>
+      <c r="C29" t="s">
+        <v>24</v>
+      </c>
+      <c r="E29" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="30" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>151</v>
+      </c>
+      <c r="B30" t="s">
         <v>152</v>
       </c>
-      <c r="E25" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>142</v>
-      </c>
-      <c r="B26" t="s">
-        <v>143</v>
-      </c>
-      <c r="C26" t="s">
-        <v>145</v>
-      </c>
-      <c r="E26" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>146</v>
-      </c>
-      <c r="B27" t="s">
-        <v>147</v>
-      </c>
-      <c r="C27" t="s">
-        <v>211</v>
-      </c>
-      <c r="E27" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>149</v>
-      </c>
-      <c r="B28" t="s">
+      <c r="C30" t="s">
+        <v>21</v>
+      </c>
+      <c r="E30" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="31" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>237</v>
+      </c>
+      <c r="B31" t="s">
+        <v>237</v>
+      </c>
+      <c r="C31" t="s">
+        <v>34</v>
+      </c>
+      <c r="E31" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="32" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>80</v>
+      </c>
+      <c r="B32" t="s">
         <v>150</v>
       </c>
-      <c r="C28" t="s">
-        <v>148</v>
-      </c>
-      <c r="E28" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>151</v>
-      </c>
-      <c r="B29" t="s">
-        <v>151</v>
-      </c>
-      <c r="C29" t="s">
-        <v>25</v>
-      </c>
-      <c r="E29" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>156</v>
-      </c>
-      <c r="B30" t="s">
-        <v>157</v>
-      </c>
-      <c r="C30" t="s">
-        <v>22</v>
-      </c>
-      <c r="E30" t="s">
+      <c r="C32" t="s">
+        <v>153</v>
+      </c>
+      <c r="E32" t="s">
         <v>63</v>
-      </c>
-    </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>203</v>
-      </c>
-      <c r="B31" t="s">
-        <v>203</v>
-      </c>
-      <c r="C31" t="s">
-        <v>13</v>
-      </c>
-      <c r="E31" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>82</v>
-      </c>
-      <c r="B32" t="s">
-        <v>155</v>
-      </c>
-      <c r="C32" t="s">
-        <v>158</v>
-      </c>
-      <c r="E32" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B33" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="C33" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="E33" t="s">
-        <v>208</v>
+        <v>198</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="B34" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="C34" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="B35" t="s">
-        <v>168</v>
+        <v>227</v>
       </c>
       <c r="C35" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="E35" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B36" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C36" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E36" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="B37" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="C37" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="B38" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="C38" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="E38" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="B39" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="C39" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E39" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="B40" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="C40" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>202</v>
+      </c>
+      <c r="B41" t="s">
+        <v>208</v>
+      </c>
+      <c r="C41" t="s">
+        <v>209</v>
+      </c>
       <c r="E41" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>217</v>
+      </c>
+      <c r="B42" t="s">
+        <v>217</v>
+      </c>
+      <c r="C42" t="s">
+        <v>28</v>
+      </c>
+      <c r="E42" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>216</v>
+      </c>
+      <c r="B43" t="s">
+        <v>218</v>
+      </c>
+      <c r="C43" t="s">
+        <v>219</v>
+      </c>
+      <c r="E43" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="E42" t="s">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>224</v>
+      </c>
+      <c r="B44" t="s">
+        <v>224</v>
+      </c>
+      <c r="C44" t="s">
+        <v>16</v>
+      </c>
+      <c r="E44" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="E43" t="s">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>223</v>
+      </c>
+      <c r="B45" t="s">
+        <v>226</v>
+      </c>
+      <c r="C45" t="s">
+        <v>228</v>
+      </c>
+      <c r="E45" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="E44" t="s">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>231</v>
+      </c>
+      <c r="B46" t="s">
+        <v>231</v>
+      </c>
+      <c r="C46" t="s">
+        <v>169</v>
+      </c>
+      <c r="E46" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="E45" t="s">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>232</v>
+      </c>
+      <c r="B47" t="s">
+        <v>233</v>
+      </c>
+      <c r="C47" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>193</v>
+      </c>
+      <c r="B48" t="s">
+        <v>239</v>
+      </c>
+      <c r="C48" t="s">
+        <v>238</v>
+      </c>
+      <c r="E48" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="E46" t="s">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>242</v>
+      </c>
+      <c r="B49" t="s">
+        <v>242</v>
+      </c>
+      <c r="C49" t="s">
+        <v>42</v>
+      </c>
+      <c r="E49" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="E48" t="s">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>243</v>
+      </c>
+      <c r="B50" t="s">
+        <v>244</v>
+      </c>
+      <c r="C50" t="s">
+        <v>245</v>
+      </c>
+      <c r="E50" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>258</v>
+      </c>
+      <c r="B51" t="s">
+        <v>258</v>
+      </c>
+      <c r="C51" t="s">
+        <v>20</v>
+      </c>
+      <c r="E51" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="49" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E49" t="s">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>260</v>
+      </c>
+      <c r="B52" t="s">
+        <v>261</v>
+      </c>
+      <c r="C52" t="s">
+        <v>259</v>
+      </c>
+      <c r="E52" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>263</v>
+      </c>
+      <c r="B53" t="s">
+        <v>264</v>
+      </c>
+      <c r="C53" t="s">
+        <v>262</v>
+      </c>
+      <c r="E53" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="50" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E50" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="51" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E51" t="s">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E54" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="52" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E52" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="53" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E53" t="s">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E55" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E56" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E57" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E58" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E60" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E61" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="54" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E54" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="55" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E55" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="56" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E56" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="57" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E57" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="58" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E58" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="60" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E60" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="61" spans="5:5" x14ac:dyDescent="0.3">
-      <c r="E61" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="62" spans="5:5" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E62" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="64" spans="5:5" x14ac:dyDescent="0.3">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="E64" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deployed 4a1c84d with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/Buch Bayrische Nächte/Sprache der Hölle.xlsx
+++ b/Buch Bayrische Nächte/Sprache der Hölle.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian Dauner\Documents\GitHub\pnpWiki\docs\Buch Bayrische Nächte\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6759AE87-4DC4-43B4-B9BC-7C0DD022F44E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8236C155-93F9-43E3-98C0-B20CBF647B47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="5205" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="707" uniqueCount="342">
   <si>
     <t>Höllisch</t>
   </si>
@@ -729,15 +729,9 @@
     <t xml:space="preserve">        -Rish</t>
   </si>
   <si>
-    <t xml:space="preserve">Nir-Ay Nir-Tra-Va-Raa </t>
-  </si>
-  <si>
     <t>many Fear</t>
   </si>
   <si>
-    <t>The seventh is Hetfoshkar and fury is his lordship</t>
-  </si>
-  <si>
     <t>The sixth is Mofylkar that is the singer of sorrows</t>
   </si>
   <si>
@@ -795,12 +789,6 @@
     <t>Ownership + Endung (Ziel)</t>
   </si>
   <si>
-    <t>Ish-Ay Ish-Foy-Tuh-Mi Ke-Mirr Vir Tra Kvo-To-Kar Tra-Osh Mi-Rof-Osh Foy Ish</t>
-  </si>
-  <si>
-    <t>Ket-Ay Ket-Foy-Fer-Ref Shat-Erk Tra-Kor Ket</t>
-  </si>
-  <si>
     <t>Curse</t>
   </si>
   <si>
@@ -832,6 +820,237 @@
   </si>
   <si>
     <t>Va-Fey</t>
+  </si>
+  <si>
+    <t>Neglectfull</t>
+  </si>
+  <si>
+    <t>neglectfull</t>
+  </si>
+  <si>
+    <t>to lead</t>
+  </si>
+  <si>
+    <t>command over</t>
+  </si>
+  <si>
+    <t>Shat-Tra-Ay</t>
+  </si>
+  <si>
+    <t>Lustfull</t>
+  </si>
+  <si>
+    <t>Lecherous</t>
+  </si>
+  <si>
+    <t>Saa-Taa-Osh</t>
+  </si>
+  <si>
+    <t>Nir-Taa-Osh</t>
+  </si>
+  <si>
+    <t>Retinue</t>
+  </si>
+  <si>
+    <t>Group of People</t>
+  </si>
+  <si>
+    <t>Oor-Mi</t>
+  </si>
+  <si>
+    <t>Saa-Ay Saa-Tra-Kar To Saa-Taa-Osh Rish Esh Tra Oor-Mi</t>
+  </si>
+  <si>
+    <t>Nir-Ay Nir-Tra-Va-Raa Shat-Tra-Mirr To Kor Nir-Taa-Osh</t>
+  </si>
+  <si>
+    <t>to say</t>
+  </si>
+  <si>
+    <t>Voice</t>
+  </si>
+  <si>
+    <t>Word</t>
+  </si>
+  <si>
+    <t>Name Haver</t>
+  </si>
+  <si>
+    <t>Name saying</t>
+  </si>
+  <si>
+    <t>Ike-Tra-Kor</t>
+  </si>
+  <si>
+    <t>Word making</t>
+  </si>
+  <si>
+    <t>make</t>
+  </si>
+  <si>
+    <t>Ike-Tra-Kaf-Kor</t>
+  </si>
+  <si>
+    <t>to sing</t>
+  </si>
+  <si>
+    <t>Word maker</t>
+  </si>
+  <si>
+    <t>Singer</t>
+  </si>
+  <si>
+    <t>Ike-Tra-Kaf-Esh</t>
+  </si>
+  <si>
+    <t>Mo-Ay Mo-Foy-Lo-Kar Erk Ike-Tra-Kaf-Esh Tra Mo-Kar</t>
+  </si>
+  <si>
+    <t>Ket-Ay Ket-Foy-Fer-Ref Shat-Erk Tra-Kor Ket-Kor</t>
+  </si>
+  <si>
+    <t>Ish-Ay Ish-Foy-Tuh-Mi Ke-Mirr Kor Tra Kvo-To-Kar Tra-Osh Mi-Rof-Osh Foy Ish-Kor</t>
+  </si>
+  <si>
+    <t>Kash-Ay Kash-Tra-Veek-Kar To Tra-Erk To Esh Kash-Osh</t>
+  </si>
+  <si>
+    <t>Ownership</t>
+  </si>
+  <si>
+    <t>The seventh is Hetfoshkar and fury is his ownership</t>
+  </si>
+  <si>
+    <t>Ke-Ay-Kor</t>
+  </si>
+  <si>
+    <t>Reign</t>
+  </si>
+  <si>
+    <t>Sum</t>
+  </si>
+  <si>
+    <t>All together</t>
+  </si>
+  <si>
+    <t>Nai-Oor</t>
+  </si>
+  <si>
+    <t>To Nai-Ay Kat Nai-Oor Foy Nai-Kar</t>
+  </si>
+  <si>
+    <t>Tuh-Ru-Osh</t>
+  </si>
+  <si>
+    <t>the Damned</t>
+  </si>
+  <si>
+    <t>Suffering Souls</t>
+  </si>
+  <si>
+    <t>Ru-Osh Tra Tuh-Ru-Osh Rish-Ri Esh Tra Shat</t>
+  </si>
+  <si>
+    <t>Rest</t>
+  </si>
+  <si>
+    <t>No Sum</t>
+  </si>
+  <si>
+    <t>Va-Nai-Oor</t>
+  </si>
+  <si>
+    <t>every</t>
+  </si>
+  <si>
+    <t>many many many</t>
+  </si>
+  <si>
+    <t>Krik-Ref</t>
+  </si>
+  <si>
+    <t>Part</t>
+  </si>
+  <si>
+    <t>To Fey-Erk-Ri Va-Nai-Oor-Kor Krik-Ref Iv-Kar Foy Ru-Kor</t>
+  </si>
+  <si>
+    <t>Het-Ay Het-Foy-Shi-Kar To Het-Kor Mirr Esh Tra Ke-Ay-Kor</t>
+  </si>
+  <si>
+    <t>to laud</t>
+  </si>
+  <si>
+    <t>to praise</t>
+  </si>
+  <si>
+    <t>no cursing</t>
+  </si>
+  <si>
+    <t>Ike- Verb</t>
+  </si>
+  <si>
+    <t>Va-Fey + Verb</t>
+  </si>
+  <si>
+    <t>Ike-Tra-Kaf + Verb</t>
+  </si>
+  <si>
+    <t>no cursing more</t>
+  </si>
+  <si>
+    <t>Va-Fey-Tat + Verb</t>
+  </si>
+  <si>
+    <t>Esh Tra Shash-Kor Mirr-Ri Foy Va-Fey-Tat-Fey</t>
+  </si>
+  <si>
+    <t>sacred</t>
+  </si>
+  <si>
+    <t>no cursed</t>
+  </si>
+  <si>
+    <t>Va-Fey-Taa</t>
+  </si>
+  <si>
+    <t>so</t>
+  </si>
+  <si>
+    <t>Do</t>
+  </si>
+  <si>
+    <t>Erk Tra Ike-Kor Mirr Va-Fey-Tat Kfo Va-Mi-Esh Ratt-Rish Tsh-Rish</t>
+  </si>
+  <si>
+    <t>Kfo Ike-Fey-Ri Nai</t>
+  </si>
+  <si>
+    <t>Daughter</t>
+  </si>
+  <si>
+    <t>small female person of</t>
+  </si>
+  <si>
+    <t>Mi-Rof-Kor Foy</t>
+  </si>
+  <si>
+    <t>Ikt-Ike-Tra-Kor</t>
+  </si>
+  <si>
+    <t>Body Word</t>
+  </si>
+  <si>
+    <t>Writing</t>
+  </si>
+  <si>
+    <t>List</t>
+  </si>
+  <si>
+    <t>many Body Word</t>
+  </si>
+  <si>
+    <t>Krik-Ikt-Ike-Tra-Kor</t>
   </si>
 </sst>
 </file>
@@ -1361,13 +1580,13 @@
     <col min="5" max="5" width="18.88671875" customWidth="1"/>
     <col min="6" max="6" width="18.33203125" customWidth="1"/>
     <col min="9" max="9" width="15.21875" customWidth="1"/>
-    <col min="11" max="11" width="10.44140625" customWidth="1"/>
+    <col min="11" max="11" width="11" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="10" customWidth="1"/>
     <col min="16" max="16" width="11.33203125" customWidth="1"/>
     <col min="18" max="18" width="11.21875" customWidth="1"/>
     <col min="19" max="19" width="17" customWidth="1"/>
     <col min="20" max="20" width="12.33203125" customWidth="1"/>
-    <col min="21" max="21" width="9.6640625" customWidth="1"/>
+    <col min="21" max="21" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="13.5546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1515,7 +1734,7 @@
         <v>150</v>
       </c>
       <c r="U3" s="7" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
     </row>
     <row r="4" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1616,7 +1835,7 @@
         <v>185</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="I6" s="6" t="s">
         <v>193</v>
@@ -1634,10 +1853,10 @@
         <v>34</v>
       </c>
       <c r="N6" s="6" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="P6" s="6" t="s">
         <v>196</v>
@@ -1645,9 +1864,15 @@
       <c r="Q6" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="R6" s="6"/>
-      <c r="S6" s="6"/>
-      <c r="T6" s="6"/>
+      <c r="R6" s="6" t="s">
+        <v>286</v>
+      </c>
+      <c r="S6" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="T6" s="6" t="s">
+        <v>330</v>
+      </c>
     </row>
     <row r="7" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
@@ -1731,10 +1956,10 @@
     </row>
     <row r="9" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="B9" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="C9" t="s">
         <v>86</v>
@@ -1755,13 +1980,13 @@
         <v>72</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="K9" s="6" t="s">
         <v>129</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="M9" s="6" t="s">
         <v>112</v>
@@ -1769,18 +1994,20 @@
       <c r="N9" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="O9" s="6"/>
+      <c r="O9" s="6" t="s">
+        <v>314</v>
+      </c>
       <c r="P9" s="6" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="Q9" s="6" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="R9" s="6" t="s">
         <v>145</v>
       </c>
       <c r="S9" s="6" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="T9" s="6" t="s">
         <v>197</v>
@@ -1856,7 +2083,7 @@
         <v>88</v>
       </c>
       <c r="C12" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E12" s="8" t="s">
         <v>202</v>
@@ -1888,7 +2115,7 @@
         <v>162</v>
       </c>
       <c r="B13" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C13" t="s">
         <v>163</v>
@@ -1907,7 +2134,7 @@
         <v>69</v>
       </c>
       <c r="B14" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C14" t="s">
         <v>95</v>
@@ -1918,7 +2145,7 @@
         <v>124</v>
       </c>
       <c r="B15" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C15" t="s">
         <v>158</v>
@@ -1932,10 +2159,10 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B16" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="C16" t="s">
         <v>155</v>
@@ -1952,7 +2179,7 @@
         <v>149</v>
       </c>
       <c r="B17" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="C17" t="s">
         <v>152</v>
@@ -1966,7 +2193,7 @@
         <v>144</v>
       </c>
       <c r="B18" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C18" t="s">
         <v>146</v>
@@ -1995,7 +2222,7 @@
         <v>92</v>
       </c>
       <c r="B19" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C19" t="s">
         <v>130</v>
@@ -2030,7 +2257,7 @@
         <v>131</v>
       </c>
       <c r="B20" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C20" t="s">
         <v>137</v>
@@ -2062,7 +2289,7 @@
         <v>98</v>
       </c>
       <c r="B21" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="C21" t="s">
         <v>97</v>
@@ -2091,13 +2318,13 @@
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
+        <v>259</v>
+      </c>
+      <c r="B22" t="s">
         <v>263</v>
       </c>
-      <c r="B22" t="s">
-        <v>267</v>
-      </c>
       <c r="C22" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="E22" t="s">
         <v>45</v>
@@ -2122,6 +2349,15 @@
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>265</v>
+      </c>
+      <c r="B23" t="s">
+        <v>266</v>
+      </c>
+      <c r="C23" t="s">
+        <v>272</v>
+      </c>
       <c r="N23" t="s">
         <v>101</v>
       </c>
@@ -2142,6 +2378,15 @@
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>267</v>
+      </c>
+      <c r="B24" t="s">
+        <v>268</v>
+      </c>
+      <c r="C24" t="s">
+        <v>269</v>
+      </c>
       <c r="E24" t="s">
         <v>46</v>
       </c>
@@ -2165,6 +2410,15 @@
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>271</v>
+      </c>
+      <c r="B25" t="s">
+        <v>270</v>
+      </c>
+      <c r="C25" t="s">
+        <v>273</v>
+      </c>
       <c r="E25" t="s">
         <v>47</v>
       </c>
@@ -2188,6 +2442,15 @@
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>274</v>
+      </c>
+      <c r="B26" t="s">
+        <v>275</v>
+      </c>
+      <c r="C26" t="s">
+        <v>276</v>
+      </c>
       <c r="E26" t="s">
         <v>48</v>
       </c>
@@ -2211,16 +2474,43 @@
       </c>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>279</v>
+      </c>
+      <c r="B27" t="s">
+        <v>283</v>
+      </c>
+      <c r="C27" t="s">
+        <v>320</v>
+      </c>
       <c r="E27" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>281</v>
+      </c>
+      <c r="B28" t="s">
+        <v>282</v>
+      </c>
+      <c r="C28" t="s">
+        <v>284</v>
+      </c>
       <c r="E28" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>280</v>
+      </c>
+      <c r="B29" t="s">
+        <v>289</v>
+      </c>
+      <c r="C29" t="s">
+        <v>287</v>
+      </c>
       <c r="E29" t="s">
         <v>51</v>
       </c>
@@ -2229,6 +2519,15 @@
       </c>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>288</v>
+      </c>
+      <c r="B30" t="s">
+        <v>285</v>
+      </c>
+      <c r="C30" t="s">
+        <v>322</v>
+      </c>
       <c r="E30" t="s">
         <v>52</v>
       </c>
@@ -2236,18 +2535,36 @@
         <v>1</v>
       </c>
       <c r="N30" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>290</v>
+      </c>
+      <c r="B31" t="s">
+        <v>290</v>
+      </c>
+      <c r="C31" t="s">
+        <v>291</v>
+      </c>
       <c r="E31" t="s">
         <v>53</v>
       </c>
       <c r="N31" t="s">
-        <v>256</v>
+        <v>294</v>
       </c>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>296</v>
+      </c>
+      <c r="B32" t="s">
+        <v>299</v>
+      </c>
+      <c r="C32" t="s">
+        <v>298</v>
+      </c>
       <c r="E32" t="s">
         <v>54</v>
       </c>
@@ -2255,18 +2572,36 @@
         <v>2</v>
       </c>
       <c r="N32" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="33" spans="5:14" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>300</v>
+      </c>
+      <c r="B33" t="s">
+        <v>301</v>
+      </c>
+      <c r="C33" t="s">
+        <v>302</v>
+      </c>
       <c r="E33" t="s">
         <v>55</v>
       </c>
       <c r="N33" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="34" spans="5:14" x14ac:dyDescent="0.3">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>305</v>
+      </c>
+      <c r="B34" t="s">
+        <v>306</v>
+      </c>
+      <c r="C34" t="s">
+        <v>304</v>
+      </c>
       <c r="E34" t="s">
         <v>56</v>
       </c>
@@ -2274,18 +2609,36 @@
         <v>3</v>
       </c>
       <c r="N34" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="35" spans="5:14" x14ac:dyDescent="0.3">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>308</v>
+      </c>
+      <c r="B35" t="s">
+        <v>309</v>
+      </c>
+      <c r="C35" t="s">
+        <v>310</v>
+      </c>
       <c r="E35" t="s">
         <v>233</v>
       </c>
       <c r="N35" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="36" spans="5:14" x14ac:dyDescent="0.3">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>311</v>
+      </c>
+      <c r="B36" t="s">
+        <v>312</v>
+      </c>
+      <c r="C36" t="s">
+        <v>313</v>
+      </c>
       <c r="E36" t="s">
         <v>57</v>
       </c>
@@ -2293,34 +2646,70 @@
         <v>4</v>
       </c>
       <c r="N36" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="37" spans="5:14" x14ac:dyDescent="0.3">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>318</v>
+      </c>
+      <c r="B37" t="s">
+        <v>319</v>
+      </c>
+      <c r="C37" t="s">
+        <v>321</v>
+      </c>
       <c r="E37" t="s">
         <v>127</v>
       </c>
       <c r="N37" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="38" spans="5:14" x14ac:dyDescent="0.3">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>317</v>
+      </c>
+      <c r="B38" t="s">
+        <v>323</v>
+      </c>
+      <c r="C38" t="s">
+        <v>324</v>
+      </c>
       <c r="M38">
         <v>5</v>
       </c>
       <c r="N38" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="39" spans="5:14" x14ac:dyDescent="0.3">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>326</v>
+      </c>
+      <c r="B39" t="s">
+        <v>327</v>
+      </c>
+      <c r="C39" t="s">
+        <v>328</v>
+      </c>
       <c r="E39" t="s">
         <v>58</v>
       </c>
       <c r="N39" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="40" spans="5:14" x14ac:dyDescent="0.3">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>333</v>
+      </c>
+      <c r="B40" t="s">
+        <v>334</v>
+      </c>
+      <c r="C40" t="s">
+        <v>335</v>
+      </c>
       <c r="E40" t="s">
         <v>59</v>
       </c>
@@ -2328,15 +2717,33 @@
         <v>6</v>
       </c>
       <c r="N40" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="41" spans="5:14" x14ac:dyDescent="0.3">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>338</v>
+      </c>
+      <c r="B41" t="s">
+        <v>337</v>
+      </c>
+      <c r="C41" t="s">
+        <v>336</v>
+      </c>
       <c r="N41" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="42" spans="5:14" x14ac:dyDescent="0.3">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>339</v>
+      </c>
+      <c r="B42" t="s">
+        <v>340</v>
+      </c>
+      <c r="C42" t="s">
+        <v>341</v>
+      </c>
       <c r="E42" t="s">
         <v>60</v>
       </c>
@@ -2344,18 +2751,18 @@
         <v>7</v>
       </c>
       <c r="N42" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="43" spans="5:14" x14ac:dyDescent="0.3">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="E43" t="s">
         <v>61</v>
       </c>
       <c r="N43" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="44" spans="5:14" x14ac:dyDescent="0.3">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
       <c r="M44">
         <v>8</v>
       </c>
@@ -2363,12 +2770,15 @@
         <v>176</v>
       </c>
     </row>
-    <row r="45" spans="5:14" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="E45" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="46" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="N45" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="E46" t="s">
         <v>63</v>
       </c>
@@ -2376,12 +2786,15 @@
         <v>177</v>
       </c>
     </row>
-    <row r="47" spans="5:14" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="E47" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="48" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="N47" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
       <c r="E48" t="s">
         <v>65</v>
       </c>
@@ -2393,6 +2806,9 @@
       <c r="E49" t="s">
         <v>66</v>
       </c>
+      <c r="N49" t="s">
+        <v>315</v>
+      </c>
     </row>
     <row r="50" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E50" t="s">
@@ -2402,6 +2818,11 @@
         <v>179</v>
       </c>
     </row>
+    <row r="51" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="N51" t="s">
+        <v>325</v>
+      </c>
+    </row>
     <row r="52" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E52" t="s">
         <v>89</v>
@@ -2414,6 +2835,9 @@
       <c r="E53" t="s">
         <v>68</v>
       </c>
+      <c r="N53" t="s">
+        <v>331</v>
+      </c>
     </row>
     <row r="54" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E54" t="s">
@@ -2421,6 +2845,11 @@
       </c>
       <c r="N54" t="s">
         <v>181</v>
+      </c>
+    </row>
+    <row r="55" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="N55" t="s">
+        <v>332</v>
       </c>
     </row>
     <row r="56" spans="5:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Deployed dc3c154 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/Buch Bayrische Nächte/Sprache der Hölle.xlsx
+++ b/Buch Bayrische Nächte/Sprache der Hölle.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian Dauner\Documents\GitHub\pnpWiki\docs\Buch Bayrische Nächte\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8236C155-93F9-43E3-98C0-B20CBF647B47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7CEE795-1CD7-47F0-AD13-D3A5D5F1ED52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5205" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="707" uniqueCount="342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="342">
   <si>
     <t>Höllisch</t>
   </si>
@@ -1014,15 +1014,9 @@
     <t>Va-Fey-Taa</t>
   </si>
   <si>
-    <t>so</t>
-  </si>
-  <si>
     <t>Do</t>
   </si>
   <si>
-    <t>Erk Tra Ike-Kor Mirr Va-Fey-Tat Kfo Va-Mi-Esh Ratt-Rish Tsh-Rish</t>
-  </si>
-  <si>
     <t>Kfo Ike-Fey-Ri Nai</t>
   </si>
   <si>
@@ -1051,6 +1045,12 @@
   </si>
   <si>
     <t>Krik-Ikt-Ike-Tra-Kor</t>
+  </si>
+  <si>
+    <t>Erk Tra Ike-Kor Mirr Va-Fey-Tat Krik Va-Mi-Esh Ratt-Rish Tsh-Rish</t>
+  </si>
+  <si>
+    <t>Movement</t>
   </si>
 </sst>
 </file>
@@ -1868,10 +1868,10 @@
         <v>286</v>
       </c>
       <c r="S6" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="T6" s="6" t="s">
         <v>329</v>
-      </c>
-      <c r="T6" s="6" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="7" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2702,13 +2702,13 @@
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
+        <v>331</v>
+      </c>
+      <c r="B40" t="s">
+        <v>332</v>
+      </c>
+      <c r="C40" t="s">
         <v>333</v>
-      </c>
-      <c r="B40" t="s">
-        <v>334</v>
-      </c>
-      <c r="C40" t="s">
-        <v>335</v>
       </c>
       <c r="E40" t="s">
         <v>59</v>
@@ -2722,13 +2722,13 @@
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="B41" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C41" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="N41" t="s">
         <v>292</v>
@@ -2736,13 +2736,13 @@
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
+        <v>337</v>
+      </c>
+      <c r="B42" t="s">
+        <v>338</v>
+      </c>
+      <c r="C42" t="s">
         <v>339</v>
-      </c>
-      <c r="B42" t="s">
-        <v>340</v>
-      </c>
-      <c r="C42" t="s">
-        <v>341</v>
       </c>
       <c r="E42" t="s">
         <v>60</v>
@@ -2836,7 +2836,7 @@
         <v>68</v>
       </c>
       <c r="N53" t="s">
-        <v>331</v>
+        <v>340</v>
       </c>
     </row>
     <row r="54" spans="5:14" x14ac:dyDescent="0.3">
@@ -2849,7 +2849,7 @@
     </row>
     <row r="55" spans="5:14" x14ac:dyDescent="0.3">
       <c r="N55" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="56" spans="5:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Deployed 27a9a8b with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/Buch Bayrische Nächte/Sprache der Hölle.xlsx
+++ b/Buch Bayrische Nächte/Sprache der Hölle.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian Dauner\Documents\GitHub\pnpWiki\docs\Buch Bayrische Nächte\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7CEE795-1CD7-47F0-AD13-D3A5D5F1ED52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BE53BA5-2E0F-4390-A5B6-9DCC7A676FA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="5205" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="345">
   <si>
     <t>Höllisch</t>
   </si>
@@ -390,9 +390,6 @@
     <t>(kein Anagramm)</t>
   </si>
   <si>
-    <t>Avarice in Loss</t>
-  </si>
-  <si>
     <t>Lust</t>
   </si>
   <si>
@@ -456,9 +453,6 @@
     <t>Sorrow out of Death</t>
   </si>
   <si>
-    <t>Anger out of Dread</t>
-  </si>
-  <si>
     <t>Hunger</t>
   </si>
   <si>
@@ -642,9 +636,6 @@
     <t>4/Envy</t>
   </si>
   <si>
-    <t>5/avarice</t>
-  </si>
-  <si>
     <t>6/Sorrow</t>
   </si>
   <si>
@@ -747,12 +738,6 @@
     <t>The first is Ishfotum that reigns in her malice over the children of pride</t>
   </si>
   <si>
-    <t>many Time</t>
-  </si>
-  <si>
-    <t>many few</t>
-  </si>
-  <si>
     <t>Doubt</t>
   </si>
   <si>
@@ -966,15 +951,9 @@
     <t>many many many</t>
   </si>
   <si>
-    <t>Krik-Ref</t>
-  </si>
-  <si>
     <t>Part</t>
   </si>
   <si>
-    <t>To Fey-Erk-Ri Va-Nai-Oor-Kor Krik-Ref Iv-Kar Foy Ru-Kor</t>
-  </si>
-  <si>
     <t>Het-Ay Het-Foy-Shi-Kar To Het-Kor Mirr Esh Tra Ke-Ay-Kor</t>
   </si>
   <si>
@@ -1044,13 +1023,43 @@
     <t>many Body Word</t>
   </si>
   <si>
-    <t>Krik-Ikt-Ike-Tra-Kor</t>
-  </si>
-  <si>
-    <t>Erk Tra Ike-Kor Mirr Va-Fey-Tat Krik Va-Mi-Esh Ratt-Rish Tsh-Rish</t>
-  </si>
-  <si>
     <t>Movement</t>
+  </si>
+  <si>
+    <t>Anger in Dread</t>
+  </si>
+  <si>
+    <t>Avarice out of Loss</t>
+  </si>
+  <si>
+    <t>fear ending</t>
+  </si>
+  <si>
+    <t>Time Ending</t>
+  </si>
+  <si>
+    <t>Veek-Ref</t>
+  </si>
+  <si>
+    <t>Veek-Ikt-Ike-Tra-Kor</t>
+  </si>
+  <si>
+    <t>To Fey-Erk-Ri Va-Nai-Oor-Kor Veek-Ref Iv-Kar Foy Ru-Kor</t>
+  </si>
+  <si>
+    <t>Erk Tra Ike-Kor Mirr Va-Fey-Tat Va-Mi-Esh Ratt-Rish Tsh-Rish</t>
+  </si>
+  <si>
+    <t>5/Avarice</t>
+  </si>
+  <si>
+    <t>Blood</t>
+  </si>
+  <si>
+    <t>Ikt-Ru</t>
+  </si>
+  <si>
+    <t>Soulf o Body</t>
   </si>
 </sst>
 </file>
@@ -1621,10 +1630,10 @@
     </row>
     <row r="2" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C2" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="E2" s="10" t="s">
         <v>32</v>
@@ -1657,10 +1666,10 @@
         <v>93</v>
       </c>
       <c r="O2" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="P2" s="11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="Q2" s="11" t="s">
         <v>10</v>
@@ -1672,7 +1681,7 @@
         <v>31</v>
       </c>
       <c r="T2" s="11" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="U2" s="12" t="s">
         <v>38</v>
@@ -1680,69 +1689,69 @@
     </row>
     <row r="3" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C3" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="G3" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="F3" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="G3" s="4" t="s">
+      <c r="H3" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="H3" s="4" t="s">
-        <v>186</v>
-      </c>
       <c r="I3" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="O3" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="P3" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="Q3" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="J3" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>189</v>
-      </c>
-      <c r="L3" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="M3" s="4" t="s">
-        <v>228</v>
-      </c>
-      <c r="N3" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="O3" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="P3" s="4" t="s">
-        <v>232</v>
-      </c>
-      <c r="Q3" s="4" t="s">
-        <v>194</v>
-      </c>
       <c r="R3" s="6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="S3" s="6" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="T3" s="6" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="U3" s="7" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
     </row>
     <row r="4" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C4" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="E4" s="15"/>
       <c r="F4" s="16"/>
@@ -1764,10 +1773,10 @@
     </row>
     <row r="5" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="C5" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>39</v>
@@ -1782,7 +1791,7 @@
         <v>13</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J5" s="11" t="s">
         <v>14</v>
@@ -1791,13 +1800,13 @@
         <v>15</v>
       </c>
       <c r="L5" s="11" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="M5" s="11" t="s">
         <v>34</v>
       </c>
       <c r="N5" s="11" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="O5" s="11" t="s">
         <v>35</v>
@@ -1820,31 +1829,31 @@
     </row>
     <row r="6" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
+        <v>219</v>
+      </c>
+      <c r="C6" t="s">
+        <v>209</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="C6" t="s">
-        <v>212</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>225</v>
-      </c>
       <c r="F6" s="3" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="J6" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="K6" s="6" t="s">
         <v>188</v>
-      </c>
-      <c r="K6" s="6" t="s">
-        <v>190</v>
       </c>
       <c r="L6" s="6" t="s">
         <v>91</v>
@@ -1853,33 +1862,33 @@
         <v>34</v>
       </c>
       <c r="N6" s="6" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="P6" s="6" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="Q6" s="6" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="R6" s="6" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="S6" s="6" t="s">
-        <v>341</v>
+        <v>332</v>
       </c>
       <c r="T6" s="6" t="s">
-        <v>329</v>
+        <v>322</v>
       </c>
     </row>
     <row r="7" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C7" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="E7" s="18"/>
       <c r="F7" s="19"/>
@@ -1900,10 +1909,10 @@
     </row>
     <row r="8" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C8" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>16</v>
@@ -1930,7 +1939,7 @@
         <v>104</v>
       </c>
       <c r="M8" s="11" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="N8" s="11" t="s">
         <v>21</v>
@@ -1956,19 +1965,19 @@
     </row>
     <row r="9" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="B9" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="C9" t="s">
         <v>86</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="G9" s="6" t="s">
         <v>94</v>
@@ -1980,37 +1989,37 @@
         <v>72</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="M9" s="6" t="s">
         <v>112</v>
       </c>
       <c r="N9" s="6" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="O9" s="6" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="P9" s="6" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="Q9" s="6" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="R9" s="6" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="S9" s="6" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="T9" s="6" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="10" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2066,13 +2075,13 @@
         <v>99</v>
       </c>
       <c r="J11" s="14" t="s">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="K11" s="14" t="s">
         <v>79</v>
       </c>
       <c r="L11" s="11" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2083,42 +2092,42 @@
         <v>88</v>
       </c>
       <c r="C12" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="E12" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="H12" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="I12" s="9" t="s">
         <v>202</v>
       </c>
-      <c r="F12" s="9" t="s">
-        <v>201</v>
-      </c>
-      <c r="G12" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="H12" s="9" t="s">
+      <c r="J12" s="9" t="s">
+        <v>341</v>
+      </c>
+      <c r="K12" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="I12" s="9" t="s">
+      <c r="L12" s="9" t="s">
         <v>204</v>
-      </c>
-      <c r="J12" s="9" t="s">
-        <v>205</v>
-      </c>
-      <c r="K12" s="9" t="s">
-        <v>206</v>
-      </c>
-      <c r="L12" s="9" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="13" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B13" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="C13" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="E13" s="20"/>
       <c r="F13" s="21"/>
@@ -2134,7 +2143,7 @@
         <v>69</v>
       </c>
       <c r="B14" t="s">
-        <v>240</v>
+        <v>336</v>
       </c>
       <c r="C14" t="s">
         <v>95</v>
@@ -2142,13 +2151,13 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B15" t="s">
-        <v>241</v>
+        <v>335</v>
       </c>
       <c r="C15" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="E15" t="s">
         <v>40</v>
@@ -2159,30 +2168,30 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="B16" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="C16" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="E16" t="s">
         <v>41</v>
       </c>
       <c r="N16" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B17" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="C17" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E17" t="s">
         <v>42</v>
@@ -2190,13 +2199,13 @@
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
+        <v>142</v>
+      </c>
+      <c r="B18" t="s">
+        <v>241</v>
+      </c>
+      <c r="C18" t="s">
         <v>144</v>
-      </c>
-      <c r="B18" t="s">
-        <v>246</v>
-      </c>
-      <c r="C18" t="s">
-        <v>146</v>
       </c>
       <c r="E18" t="s">
         <v>73</v>
@@ -2211,7 +2220,7 @@
         <v>0</v>
       </c>
       <c r="T18" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="V18" t="s">
         <v>114</v>
@@ -2222,10 +2231,10 @@
         <v>92</v>
       </c>
       <c r="B19" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="C19" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E19" t="s">
         <v>74</v>
@@ -2240,13 +2249,13 @@
         <v>117</v>
       </c>
       <c r="S19" t="s">
+        <v>137</v>
+      </c>
+      <c r="T19" t="s">
         <v>138</v>
       </c>
-      <c r="T19" t="s">
-        <v>139</v>
-      </c>
       <c r="V19" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="W19" t="s">
         <v>120</v>
@@ -2254,13 +2263,13 @@
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B20" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="C20" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E20" t="s">
         <v>43</v>
@@ -2272,16 +2281,16 @@
         <v>76</v>
       </c>
       <c r="Q20" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="S20" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="T20" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="V20" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.3">
@@ -2289,7 +2298,7 @@
         <v>98</v>
       </c>
       <c r="B21" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="C21" t="s">
         <v>97</v>
@@ -2298,33 +2307,33 @@
         <v>44</v>
       </c>
       <c r="N21" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="O21" t="s">
         <v>77</v>
       </c>
       <c r="Q21" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="S21" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="T21" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="V21" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
+        <v>254</v>
+      </c>
+      <c r="B22" t="s">
+        <v>258</v>
+      </c>
+      <c r="C22" t="s">
         <v>259</v>
-      </c>
-      <c r="B22" t="s">
-        <v>263</v>
-      </c>
-      <c r="C22" t="s">
-        <v>264</v>
       </c>
       <c r="E22" t="s">
         <v>45</v>
@@ -2339,24 +2348,24 @@
         <v>118</v>
       </c>
       <c r="S22" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="T22" t="s">
+        <v>164</v>
+      </c>
+      <c r="V22" t="s">
         <v>166</v>
-      </c>
-      <c r="V22" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="B23" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="C23" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="N23" t="s">
         <v>101</v>
@@ -2365,27 +2374,27 @@
         <v>99</v>
       </c>
       <c r="Q23" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="S23" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="T23" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="V23" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="B24" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="C24" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="E24" t="s">
         <v>46</v>
@@ -2394,30 +2403,30 @@
         <v>102</v>
       </c>
       <c r="O24" t="s">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="Q24" t="s">
-        <v>121</v>
+        <v>334</v>
       </c>
       <c r="S24" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="T24" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="V24" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="B25" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="C25" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="E25" t="s">
         <v>47</v>
@@ -2429,27 +2438,27 @@
         <v>79</v>
       </c>
       <c r="Q25" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="S25" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="T25" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="V25" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="B26" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="C26" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="E26" t="s">
         <v>48</v>
@@ -2458,30 +2467,30 @@
         <v>103</v>
       </c>
       <c r="O26" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="Q26" t="s">
-        <v>143</v>
+        <v>333</v>
       </c>
       <c r="S26" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="T26" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="V26" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="B27" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="C27" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="E27" t="s">
         <v>49</v>
@@ -2489,13 +2498,13 @@
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="B28" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="C28" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="E28" t="s">
         <v>50</v>
@@ -2503,30 +2512,30 @@
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="B29" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="C29" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="E29" t="s">
         <v>51</v>
       </c>
       <c r="N29" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="B30" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="C30" t="s">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="E30" t="s">
         <v>52</v>
@@ -2535,35 +2544,35 @@
         <v>1</v>
       </c>
       <c r="N30" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="B31" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="C31" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="E31" t="s">
         <v>53</v>
       </c>
       <c r="N31" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="B32" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="C32" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="E32" t="s">
         <v>54</v>
@@ -2572,35 +2581,35 @@
         <v>2</v>
       </c>
       <c r="N32" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="B33" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="C33" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="E33" t="s">
         <v>55</v>
       </c>
       <c r="N33" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="B34" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="C34" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="E34" t="s">
         <v>56</v>
@@ -2609,35 +2618,35 @@
         <v>3</v>
       </c>
       <c r="N34" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="B35" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="C35" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="E35" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="N35" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="B36" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="C36" t="s">
-        <v>313</v>
+        <v>337</v>
       </c>
       <c r="E36" t="s">
         <v>57</v>
@@ -2646,69 +2655,69 @@
         <v>4</v>
       </c>
       <c r="N36" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="B37" t="s">
-        <v>319</v>
+        <v>312</v>
       </c>
       <c r="C37" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
       <c r="E37" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="N37" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
+        <v>310</v>
+      </c>
+      <c r="B38" t="s">
+        <v>316</v>
+      </c>
+      <c r="C38" t="s">
         <v>317</v>
-      </c>
-      <c r="B38" t="s">
-        <v>323</v>
-      </c>
-      <c r="C38" t="s">
-        <v>324</v>
       </c>
       <c r="M38">
         <v>5</v>
       </c>
       <c r="N38" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
       <c r="B39" t="s">
-        <v>327</v>
+        <v>320</v>
       </c>
       <c r="C39" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
       <c r="E39" t="s">
         <v>58</v>
       </c>
       <c r="N39" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>331</v>
+        <v>324</v>
       </c>
       <c r="B40" t="s">
-        <v>332</v>
+        <v>325</v>
       </c>
       <c r="C40" t="s">
-        <v>333</v>
+        <v>326</v>
       </c>
       <c r="E40" t="s">
         <v>59</v>
@@ -2717,32 +2726,32 @@
         <v>6</v>
       </c>
       <c r="N40" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>336</v>
+        <v>329</v>
       </c>
       <c r="B41" t="s">
-        <v>335</v>
+        <v>328</v>
       </c>
       <c r="C41" t="s">
-        <v>334</v>
+        <v>327</v>
       </c>
       <c r="N41" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="B42" t="s">
+        <v>331</v>
+      </c>
+      <c r="C42" t="s">
         <v>338</v>
-      </c>
-      <c r="C42" t="s">
-        <v>339</v>
       </c>
       <c r="E42" t="s">
         <v>60</v>
@@ -2751,15 +2760,24 @@
         <v>7</v>
       </c>
       <c r="N42" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>342</v>
+      </c>
+      <c r="B43" t="s">
+        <v>344</v>
+      </c>
+      <c r="C43" t="s">
+        <v>343</v>
+      </c>
       <c r="E43" t="s">
         <v>61</v>
       </c>
       <c r="N43" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.3">
@@ -2767,7 +2785,7 @@
         <v>8</v>
       </c>
       <c r="N44" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.3">
@@ -2775,7 +2793,7 @@
         <v>62</v>
       </c>
       <c r="N45" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.3">
@@ -2783,7 +2801,7 @@
         <v>63</v>
       </c>
       <c r="N46" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
@@ -2791,7 +2809,7 @@
         <v>64</v>
       </c>
       <c r="N47" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.3">
@@ -2799,7 +2817,7 @@
         <v>65</v>
       </c>
       <c r="N48" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="49" spans="5:14" x14ac:dyDescent="0.3">
@@ -2807,7 +2825,7 @@
         <v>66</v>
       </c>
       <c r="N49" t="s">
-        <v>315</v>
+        <v>339</v>
       </c>
     </row>
     <row r="50" spans="5:14" x14ac:dyDescent="0.3">
@@ -2815,12 +2833,12 @@
         <v>67</v>
       </c>
       <c r="N50" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="51" spans="5:14" x14ac:dyDescent="0.3">
       <c r="N51" t="s">
-        <v>325</v>
+        <v>318</v>
       </c>
     </row>
     <row r="52" spans="5:14" x14ac:dyDescent="0.3">
@@ -2828,7 +2846,7 @@
         <v>89</v>
       </c>
       <c r="N52" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="53" spans="5:14" x14ac:dyDescent="0.3">
@@ -2844,12 +2862,12 @@
         <v>108</v>
       </c>
       <c r="N54" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="55" spans="5:14" x14ac:dyDescent="0.3">
       <c r="N55" t="s">
-        <v>330</v>
+        <v>323</v>
       </c>
     </row>
     <row r="56" spans="5:14" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Deployed 9862510 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/Buch Bayrische Nächte/Sprache der Hölle.xlsx
+++ b/Buch Bayrische Nächte/Sprache der Hölle.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian Dauner\Documents\GitHub\pnpWiki\docs\Buch Bayrische Nächte\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BE53BA5-2E0F-4390-A5B6-9DCC7A676FA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BA8F24B-AB5D-4BB1-A540-7888679420E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="5205" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -252,9 +252,6 @@
     <t xml:space="preserve">        -Osh (Mehrzahl)</t>
   </si>
   <si>
-    <t xml:space="preserve">Das Zählsystem ist ein Eptasystem von 1-7. </t>
-  </si>
-  <si>
     <t>Ish</t>
   </si>
   <si>
@@ -1060,6 +1057,9 @@
   </si>
   <si>
     <t>Soulf o Body</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Das Zählsystem ist ein Oktontalsystem von 1-7. </t>
   </si>
 </sst>
 </file>
@@ -1630,10 +1630,10 @@
     </row>
     <row r="2" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E2" s="10" t="s">
         <v>32</v>
@@ -1663,13 +1663,13 @@
         <v>9</v>
       </c>
       <c r="N2" s="11" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="O2" s="11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="P2" s="11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="Q2" s="11" t="s">
         <v>10</v>
@@ -1681,7 +1681,7 @@
         <v>31</v>
       </c>
       <c r="T2" s="11" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="U2" s="12" t="s">
         <v>38</v>
@@ -1689,69 +1689,69 @@
     </row>
     <row r="3" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="G3" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="G3" s="4" t="s">
-        <v>182</v>
-      </c>
       <c r="H3" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="J3" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="I3" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="J3" s="4" t="s">
-        <v>185</v>
-      </c>
       <c r="K3" s="4" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="L3" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="M3" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="O3" s="4" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="P3" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="Q3" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="R3" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="S3" s="6" t="s">
         <v>228</v>
       </c>
-      <c r="Q3" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="R3" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="S3" s="6" t="s">
-        <v>229</v>
-      </c>
       <c r="T3" s="6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="U3" s="7" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="4" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E4" s="15"/>
       <c r="F4" s="16"/>
@@ -1773,10 +1773,10 @@
     </row>
     <row r="5" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>39</v>
@@ -1791,7 +1791,7 @@
         <v>13</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J5" s="11" t="s">
         <v>14</v>
@@ -1800,13 +1800,13 @@
         <v>15</v>
       </c>
       <c r="L5" s="11" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="M5" s="11" t="s">
         <v>34</v>
       </c>
       <c r="N5" s="11" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="O5" s="11" t="s">
         <v>35</v>
@@ -1815,7 +1815,7 @@
         <v>36</v>
       </c>
       <c r="Q5" s="11" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="R5" s="11" t="s">
         <v>28</v>
@@ -1829,66 +1829,66 @@
     </row>
     <row r="6" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C6" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E6" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>223</v>
-      </c>
       <c r="G6" s="6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="M6" s="6" t="s">
         <v>34</v>
       </c>
       <c r="N6" s="6" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="P6" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="Q6" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="R6" s="6" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="S6" s="6" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="T6" s="6" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="7" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E7" s="18"/>
       <c r="F7" s="19"/>
@@ -1909,10 +1909,10 @@
     </row>
     <row r="8" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C8" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>16</v>
@@ -1930,16 +1930,16 @@
         <v>20</v>
       </c>
       <c r="J8" s="11" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K8" s="11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="L8" s="11" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="M8" s="11" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="N8" s="11" t="s">
         <v>21</v>
@@ -1965,72 +1965,72 @@
     </row>
     <row r="9" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
+        <v>251</v>
+      </c>
+      <c r="B9" t="s">
         <v>252</v>
       </c>
-      <c r="B9" t="s">
-        <v>253</v>
-      </c>
       <c r="C9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I9" s="6" t="s">
         <v>72</v>
       </c>
       <c r="J9" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="L9" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="M9" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="N9" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="O9" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="P9" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="Q9" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="R9" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="S9" s="6" t="s">
         <v>244</v>
       </c>
-      <c r="K9" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="L9" s="6" t="s">
-        <v>237</v>
-      </c>
-      <c r="M9" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="N9" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="O9" s="6" t="s">
-        <v>308</v>
-      </c>
-      <c r="P9" s="6" t="s">
-        <v>251</v>
-      </c>
-      <c r="Q9" s="6" t="s">
-        <v>243</v>
-      </c>
-      <c r="R9" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="S9" s="6" t="s">
-        <v>245</v>
-      </c>
       <c r="T9" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="10" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C10" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E10" s="15"/>
       <c r="F10" s="16"/>
@@ -2051,83 +2051,83 @@
     </row>
     <row r="11" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
+        <v>82</v>
+      </c>
+      <c r="B11" t="s">
         <v>83</v>
       </c>
-      <c r="B11" t="s">
-        <v>84</v>
-      </c>
       <c r="C11" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F11" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="G11" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="G11" s="14" t="s">
+      <c r="H11" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="H11" s="14" t="s">
+      <c r="I11" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="J11" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="K11" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="I11" s="14" t="s">
+      <c r="L11" s="11" t="s">
         <v>99</v>
-      </c>
-      <c r="J11" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="K11" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="L11" s="11" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
+        <v>86</v>
+      </c>
+      <c r="B12" t="s">
         <v>87</v>
       </c>
-      <c r="B12" t="s">
-        <v>88</v>
-      </c>
       <c r="C12" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E12" s="8" t="s">
+        <v>199</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="H12" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="F12" s="9" t="s">
-        <v>199</v>
-      </c>
-      <c r="G12" s="9" t="s">
-        <v>227</v>
-      </c>
-      <c r="H12" s="9" t="s">
+      <c r="I12" s="9" t="s">
         <v>201</v>
       </c>
-      <c r="I12" s="9" t="s">
+      <c r="J12" s="9" t="s">
+        <v>340</v>
+      </c>
+      <c r="K12" s="9" t="s">
         <v>202</v>
       </c>
-      <c r="J12" s="9" t="s">
-        <v>341</v>
-      </c>
-      <c r="K12" s="9" t="s">
+      <c r="L12" s="9" t="s">
         <v>203</v>
-      </c>
-      <c r="L12" s="9" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="13" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B13" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E13" s="20"/>
       <c r="F13" s="21"/>
@@ -2143,55 +2143,55 @@
         <v>69</v>
       </c>
       <c r="B14" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C14" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B15" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C15" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E15" t="s">
         <v>40</v>
       </c>
       <c r="N15" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
+        <v>237</v>
+      </c>
+      <c r="B16" t="s">
         <v>238</v>
       </c>
-      <c r="B16" t="s">
-        <v>239</v>
-      </c>
       <c r="C16" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E16" t="s">
         <v>41</v>
       </c>
       <c r="N16" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B17" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C17" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E17" t="s">
         <v>42</v>
@@ -2199,298 +2199,298 @@
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B18" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E18" t="s">
         <v>73</v>
       </c>
       <c r="N18" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="Q18" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="S18" t="s">
         <v>0</v>
       </c>
       <c r="T18" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="V18" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B19" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C19" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E19" t="s">
         <v>74</v>
       </c>
       <c r="N19" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="O19" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="Q19" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="S19" t="s">
+        <v>136</v>
+      </c>
+      <c r="T19" t="s">
         <v>137</v>
       </c>
-      <c r="T19" t="s">
-        <v>138</v>
-      </c>
       <c r="V19" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="W19" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B20" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C20" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E20" t="s">
         <v>43</v>
       </c>
       <c r="N20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O20" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="Q20" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="S20" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="T20" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="V20" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B21" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C21" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E21" t="s">
         <v>44</v>
       </c>
       <c r="N21" t="s">
+        <v>120</v>
+      </c>
+      <c r="O21" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q21" t="s">
         <v>121</v>
       </c>
-      <c r="O21" t="s">
-        <v>77</v>
-      </c>
-      <c r="Q21" t="s">
-        <v>122</v>
-      </c>
       <c r="S21" t="s">
+        <v>144</v>
+      </c>
+      <c r="T21" t="s">
         <v>145</v>
       </c>
-      <c r="T21" t="s">
-        <v>146</v>
-      </c>
       <c r="V21" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B22" t="s">
+        <v>257</v>
+      </c>
+      <c r="C22" t="s">
         <v>258</v>
-      </c>
-      <c r="C22" t="s">
-        <v>259</v>
       </c>
       <c r="E22" t="s">
         <v>45</v>
       </c>
       <c r="N22" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="O22" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="Q22" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="S22" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="T22" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="V22" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
+        <v>259</v>
+      </c>
+      <c r="B23" t="s">
         <v>260</v>
       </c>
-      <c r="B23" t="s">
-        <v>261</v>
-      </c>
       <c r="C23" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="N23" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O23" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="Q23" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="S23" t="s">
+        <v>153</v>
+      </c>
+      <c r="T23" t="s">
         <v>154</v>
       </c>
-      <c r="T23" t="s">
-        <v>155</v>
-      </c>
       <c r="V23" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
+        <v>261</v>
+      </c>
+      <c r="B24" t="s">
         <v>262</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>263</v>
-      </c>
-      <c r="C24" t="s">
-        <v>264</v>
       </c>
       <c r="E24" t="s">
         <v>46</v>
       </c>
       <c r="N24" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="O24" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="Q24" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="S24" t="s">
+        <v>161</v>
+      </c>
+      <c r="T24" t="s">
         <v>162</v>
       </c>
-      <c r="T24" t="s">
-        <v>163</v>
-      </c>
       <c r="V24" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B25" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C25" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E25" t="s">
         <v>47</v>
       </c>
       <c r="N25" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="O25" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="Q25" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="S25" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="T25" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="V25" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
+        <v>268</v>
+      </c>
+      <c r="B26" t="s">
         <v>269</v>
       </c>
-      <c r="B26" t="s">
+      <c r="C26" t="s">
         <v>270</v>
-      </c>
-      <c r="C26" t="s">
-        <v>271</v>
       </c>
       <c r="E26" t="s">
         <v>48</v>
       </c>
       <c r="N26" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="O26" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q26" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="S26" t="s">
+        <v>156</v>
+      </c>
+      <c r="T26" t="s">
         <v>157</v>
       </c>
-      <c r="T26" t="s">
-        <v>158</v>
-      </c>
       <c r="V26" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B27" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C27" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E27" t="s">
         <v>49</v>
@@ -2498,13 +2498,13 @@
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
+        <v>275</v>
+      </c>
+      <c r="B28" t="s">
         <v>276</v>
       </c>
-      <c r="B28" t="s">
-        <v>277</v>
-      </c>
       <c r="C28" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="E28" t="s">
         <v>50</v>
@@ -2512,30 +2512,30 @@
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B29" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C29" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E29" t="s">
         <v>51</v>
       </c>
       <c r="N29" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B30" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C30" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="E30" t="s">
         <v>52</v>
@@ -2544,35 +2544,35 @@
         <v>1</v>
       </c>
       <c r="N30" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
+        <v>284</v>
+      </c>
+      <c r="B31" t="s">
+        <v>284</v>
+      </c>
+      <c r="C31" t="s">
         <v>285</v>
-      </c>
-      <c r="B31" t="s">
-        <v>285</v>
-      </c>
-      <c r="C31" t="s">
-        <v>286</v>
       </c>
       <c r="E31" t="s">
         <v>53</v>
       </c>
       <c r="N31" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B32" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C32" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="E32" t="s">
         <v>54</v>
@@ -2581,35 +2581,35 @@
         <v>2</v>
       </c>
       <c r="N32" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
+        <v>294</v>
+      </c>
+      <c r="B33" t="s">
         <v>295</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
         <v>296</v>
-      </c>
-      <c r="C33" t="s">
-        <v>297</v>
       </c>
       <c r="E33" t="s">
         <v>55</v>
       </c>
       <c r="N33" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>299</v>
+      </c>
+      <c r="B34" t="s">
         <v>300</v>
       </c>
-      <c r="B34" t="s">
-        <v>301</v>
-      </c>
       <c r="C34" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E34" t="s">
         <v>56</v>
@@ -2618,35 +2618,35 @@
         <v>3</v>
       </c>
       <c r="N34" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
+        <v>302</v>
+      </c>
+      <c r="B35" t="s">
         <v>303</v>
       </c>
-      <c r="B35" t="s">
+      <c r="C35" t="s">
         <v>304</v>
       </c>
-      <c r="C35" t="s">
-        <v>305</v>
-      </c>
       <c r="E35" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="N35" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
+        <v>305</v>
+      </c>
+      <c r="B36" t="s">
         <v>306</v>
       </c>
-      <c r="B36" t="s">
-        <v>307</v>
-      </c>
       <c r="C36" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E36" t="s">
         <v>57</v>
@@ -2655,69 +2655,69 @@
         <v>4</v>
       </c>
       <c r="N36" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
+        <v>310</v>
+      </c>
+      <c r="B37" t="s">
         <v>311</v>
       </c>
-      <c r="B37" t="s">
-        <v>312</v>
-      </c>
       <c r="C37" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E37" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="N37" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B38" t="s">
+        <v>315</v>
+      </c>
+      <c r="C38" t="s">
         <v>316</v>
-      </c>
-      <c r="C38" t="s">
-        <v>317</v>
       </c>
       <c r="M38">
         <v>5</v>
       </c>
       <c r="N38" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
+        <v>318</v>
+      </c>
+      <c r="B39" t="s">
         <v>319</v>
       </c>
-      <c r="B39" t="s">
+      <c r="C39" t="s">
         <v>320</v>
-      </c>
-      <c r="C39" t="s">
-        <v>321</v>
       </c>
       <c r="E39" t="s">
         <v>58</v>
       </c>
       <c r="N39" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
+        <v>323</v>
+      </c>
+      <c r="B40" t="s">
         <v>324</v>
       </c>
-      <c r="B40" t="s">
+      <c r="C40" t="s">
         <v>325</v>
-      </c>
-      <c r="C40" t="s">
-        <v>326</v>
       </c>
       <c r="E40" t="s">
         <v>59</v>
@@ -2726,32 +2726,32 @@
         <v>6</v>
       </c>
       <c r="N40" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="B41" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C41" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="N41" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
+        <v>329</v>
+      </c>
+      <c r="B42" t="s">
         <v>330</v>
       </c>
-      <c r="B42" t="s">
-        <v>331</v>
-      </c>
       <c r="C42" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="E42" t="s">
         <v>60</v>
@@ -2760,24 +2760,24 @@
         <v>7</v>
       </c>
       <c r="N42" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
+        <v>341</v>
+      </c>
+      <c r="B43" t="s">
+        <v>343</v>
+      </c>
+      <c r="C43" t="s">
         <v>342</v>
-      </c>
-      <c r="B43" t="s">
-        <v>344</v>
-      </c>
-      <c r="C43" t="s">
-        <v>343</v>
       </c>
       <c r="E43" t="s">
         <v>61</v>
       </c>
       <c r="N43" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.3">
@@ -2785,7 +2785,7 @@
         <v>8</v>
       </c>
       <c r="N44" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.3">
@@ -2793,7 +2793,7 @@
         <v>62</v>
       </c>
       <c r="N45" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.3">
@@ -2801,7 +2801,7 @@
         <v>63</v>
       </c>
       <c r="N46" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
@@ -2809,7 +2809,7 @@
         <v>64</v>
       </c>
       <c r="N47" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.3">
@@ -2817,7 +2817,7 @@
         <v>65</v>
       </c>
       <c r="N48" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="49" spans="5:14" x14ac:dyDescent="0.3">
@@ -2825,7 +2825,7 @@
         <v>66</v>
       </c>
       <c r="N49" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="50" spans="5:14" x14ac:dyDescent="0.3">
@@ -2833,20 +2833,20 @@
         <v>67</v>
       </c>
       <c r="N50" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="51" spans="5:14" x14ac:dyDescent="0.3">
       <c r="N51" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="52" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E52" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="N52" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="53" spans="5:14" x14ac:dyDescent="0.3">
@@ -2854,25 +2854,25 @@
         <v>68</v>
       </c>
       <c r="N53" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="54" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E54" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="N54" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="55" spans="5:14" x14ac:dyDescent="0.3">
       <c r="N55" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="56" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E56" t="s">
-        <v>75</v>
+        <v>344</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deployed 8de05b1 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/Buch Bayrische Nächte/Sprache der Hölle.xlsx
+++ b/Buch Bayrische Nächte/Sprache der Hölle.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian Dauner\Documents\GitHub\pnpWiki\docs\Buch Bayrische Nächte\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BA8F24B-AB5D-4BB1-A540-7888679420E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49C7D215-4FF9-4E4D-98AF-82CBC1EDB488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="5205" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="357" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="354">
   <si>
     <t>Höllisch</t>
   </si>
@@ -1056,10 +1056,37 @@
     <t>Ikt-Ru</t>
   </si>
   <si>
-    <t>Soulf o Body</t>
-  </si>
-  <si>
     <t xml:space="preserve">Das Zählsystem ist ein Oktontalsystem von 1-7. </t>
+  </si>
+  <si>
+    <t>Shkarhound</t>
+  </si>
+  <si>
+    <t>Anger Feeder</t>
+  </si>
+  <si>
+    <t>Food</t>
+  </si>
+  <si>
+    <t>Soulf of Body</t>
+  </si>
+  <si>
+    <t>Feeder</t>
+  </si>
+  <si>
+    <t>Fullness filling</t>
+  </si>
+  <si>
+    <t>Raa-Kor</t>
+  </si>
+  <si>
+    <t>Fullness Filler</t>
+  </si>
+  <si>
+    <t>Raa-Esh</t>
+  </si>
+  <si>
+    <t>Kash-Raa-Esh</t>
   </si>
 </sst>
 </file>
@@ -2768,7 +2795,7 @@
         <v>341</v>
       </c>
       <c r="B43" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="C43" t="s">
         <v>342</v>
@@ -2781,6 +2808,15 @@
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>142</v>
+      </c>
+      <c r="B44" t="s">
+        <v>142</v>
+      </c>
+      <c r="C44" t="s">
+        <v>25</v>
+      </c>
       <c r="M44">
         <v>8</v>
       </c>
@@ -2789,6 +2825,15 @@
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>346</v>
+      </c>
+      <c r="B45" t="s">
+        <v>349</v>
+      </c>
+      <c r="C45" t="s">
+        <v>350</v>
+      </c>
       <c r="E45" t="s">
         <v>62</v>
       </c>
@@ -2797,6 +2842,15 @@
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>348</v>
+      </c>
+      <c r="B46" t="s">
+        <v>351</v>
+      </c>
+      <c r="C46" t="s">
+        <v>352</v>
+      </c>
       <c r="E46" t="s">
         <v>63</v>
       </c>
@@ -2805,6 +2859,15 @@
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>344</v>
+      </c>
+      <c r="B47" t="s">
+        <v>345</v>
+      </c>
+      <c r="C47" t="s">
+        <v>353</v>
+      </c>
       <c r="E47" t="s">
         <v>64</v>
       </c>
@@ -2872,7 +2935,7 @@
     </row>
     <row r="56" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E56" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deployed eb1d0e2 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/Buch Bayrische Nächte/Sprache der Hölle.xlsx
+++ b/Buch Bayrische Nächte/Sprache der Hölle.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian Dauner\Documents\GitHub\pnpWiki\docs\Buch Bayrische Nächte\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49C7D215-4FF9-4E4D-98AF-82CBC1EDB488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5EC790C-5D06-4C8B-BC8D-E2D91631B918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="5205" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="369">
   <si>
     <t>Höllisch</t>
   </si>
@@ -591,9 +591,6 @@
     <t>Komperativ</t>
   </si>
   <si>
-    <t>Superaltiv</t>
-  </si>
-  <si>
     <t>They/we (male)</t>
   </si>
   <si>
@@ -1087,6 +1084,54 @@
   </si>
   <si>
     <t>Kash-Raa-Esh</t>
+  </si>
+  <si>
+    <t>Tooth</t>
+  </si>
+  <si>
+    <t>Superlativ</t>
+  </si>
+  <si>
+    <t>Mouth</t>
+  </si>
+  <si>
+    <t>Body Filler</t>
+  </si>
+  <si>
+    <t>Ikt-Raa-Esh</t>
+  </si>
+  <si>
+    <t>Body Filler Together</t>
+  </si>
+  <si>
+    <t>Ikt-Raa-Oor-Esh</t>
+  </si>
+  <si>
+    <t>to collect</t>
+  </si>
+  <si>
+    <t>together doer</t>
+  </si>
+  <si>
+    <t>Oor-Fey</t>
+  </si>
+  <si>
+    <t>Collector</t>
+  </si>
+  <si>
+    <t>Oor-Fey-Esh</t>
+  </si>
+  <si>
+    <t>together do</t>
+  </si>
+  <si>
+    <t>Markings</t>
+  </si>
+  <si>
+    <t>Ikt-Ke-Tra-Ash</t>
+  </si>
+  <si>
+    <t>Body Ashbearer</t>
   </si>
 </sst>
 </file>
@@ -1657,10 +1702,10 @@
     </row>
     <row r="2" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E2" s="10" t="s">
         <v>32</v>
@@ -1708,7 +1753,7 @@
         <v>31</v>
       </c>
       <c r="T2" s="11" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="U2" s="12" t="s">
         <v>38</v>
@@ -1716,10 +1761,10 @@
     </row>
     <row r="3" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C3" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>179</v>
@@ -1734,7 +1779,7 @@
         <v>183</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="J3" s="4" t="s">
         <v>184</v>
@@ -1743,42 +1788,42 @@
         <v>186</v>
       </c>
       <c r="L3" s="4" t="s">
-        <v>188</v>
+        <v>354</v>
       </c>
       <c r="M3" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="O3" s="4" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="Q3" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="R3" s="6" t="s">
         <v>158</v>
       </c>
       <c r="S3" s="6" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="T3" s="6" t="s">
         <v>147</v>
       </c>
       <c r="U3" s="7" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="4" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E4" s="15"/>
       <c r="F4" s="16"/>
@@ -1800,10 +1845,10 @@
     </row>
     <row r="5" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C5" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>39</v>
@@ -1833,7 +1878,7 @@
         <v>34</v>
       </c>
       <c r="N5" s="11" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="O5" s="11" t="s">
         <v>35</v>
@@ -1856,25 +1901,25 @@
     </row>
     <row r="6" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C6" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E6" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>221</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>222</v>
       </c>
       <c r="G6" s="6" t="s">
         <v>182</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="J6" s="6" t="s">
         <v>185</v>
@@ -1889,33 +1934,33 @@
         <v>34</v>
       </c>
       <c r="N6" s="6" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="P6" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="Q6" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="R6" s="6" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="S6" s="6" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="T6" s="6" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="7" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E7" s="18"/>
       <c r="F7" s="19"/>
@@ -1936,10 +1981,10 @@
     </row>
     <row r="8" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C8" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>16</v>
@@ -1966,7 +2011,7 @@
         <v>103</v>
       </c>
       <c r="M8" s="11" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="N8" s="11" t="s">
         <v>21</v>
@@ -1992,19 +2037,19 @@
     </row>
     <row r="9" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
+        <v>250</v>
+      </c>
+      <c r="B9" t="s">
         <v>251</v>
-      </c>
-      <c r="B9" t="s">
-        <v>252</v>
       </c>
       <c r="C9" t="s">
         <v>85</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="G9" s="6" t="s">
         <v>93</v>
@@ -2016,37 +2061,37 @@
         <v>72</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="K9" s="6" t="s">
         <v>127</v>
       </c>
       <c r="L9" s="6" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="M9" s="6" t="s">
         <v>111</v>
       </c>
       <c r="N9" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="O9" s="6" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="P9" s="6" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="Q9" s="6" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="R9" s="6" t="s">
         <v>142</v>
       </c>
       <c r="S9" s="6" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="T9" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="10" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2119,31 +2164,31 @@
         <v>87</v>
       </c>
       <c r="C12" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="E12" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="H12" s="9" t="s">
         <v>199</v>
       </c>
-      <c r="F12" s="9" t="s">
-        <v>198</v>
-      </c>
-      <c r="G12" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="H12" s="9" t="s">
+      <c r="I12" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="I12" s="9" t="s">
+      <c r="J12" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="K12" s="9" t="s">
         <v>201</v>
       </c>
-      <c r="J12" s="9" t="s">
-        <v>340</v>
-      </c>
-      <c r="K12" s="9" t="s">
+      <c r="L12" s="9" t="s">
         <v>202</v>
-      </c>
-      <c r="L12" s="9" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="13" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2151,7 +2196,7 @@
         <v>159</v>
       </c>
       <c r="B13" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C13" t="s">
         <v>155</v>
@@ -2170,7 +2215,7 @@
         <v>69</v>
       </c>
       <c r="B14" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C14" t="s">
         <v>94</v>
@@ -2181,7 +2226,7 @@
         <v>122</v>
       </c>
       <c r="B15" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C15" t="s">
         <v>160</v>
@@ -2195,10 +2240,10 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
+        <v>236</v>
+      </c>
+      <c r="B16" t="s">
         <v>237</v>
-      </c>
-      <c r="B16" t="s">
-        <v>238</v>
       </c>
       <c r="C16" t="s">
         <v>152</v>
@@ -2215,7 +2260,7 @@
         <v>146</v>
       </c>
       <c r="B17" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C17" t="s">
         <v>149</v>
@@ -2229,7 +2274,7 @@
         <v>141</v>
       </c>
       <c r="B18" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C18" t="s">
         <v>143</v>
@@ -2258,7 +2303,7 @@
         <v>91</v>
       </c>
       <c r="B19" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C19" t="s">
         <v>128</v>
@@ -2293,7 +2338,7 @@
         <v>129</v>
       </c>
       <c r="B20" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C20" t="s">
         <v>135</v>
@@ -2325,7 +2370,7 @@
         <v>97</v>
       </c>
       <c r="B21" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C21" t="s">
         <v>96</v>
@@ -2354,13 +2399,13 @@
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B22" t="s">
+        <v>256</v>
+      </c>
+      <c r="C22" t="s">
         <v>257</v>
-      </c>
-      <c r="C22" t="s">
-        <v>258</v>
       </c>
       <c r="E22" t="s">
         <v>45</v>
@@ -2386,13 +2431,13 @@
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
+        <v>258</v>
+      </c>
+      <c r="B23" t="s">
         <v>259</v>
       </c>
-      <c r="B23" t="s">
-        <v>260</v>
-      </c>
       <c r="C23" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="N23" t="s">
         <v>100</v>
@@ -2415,13 +2460,13 @@
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
+        <v>260</v>
+      </c>
+      <c r="B24" t="s">
         <v>261</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>262</v>
-      </c>
-      <c r="C24" t="s">
-        <v>263</v>
       </c>
       <c r="E24" t="s">
         <v>46</v>
@@ -2433,7 +2478,7 @@
         <v>79</v>
       </c>
       <c r="Q24" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="S24" t="s">
         <v>161</v>
@@ -2447,13 +2492,13 @@
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B25" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C25" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E25" t="s">
         <v>47</v>
@@ -2479,13 +2524,13 @@
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
+        <v>267</v>
+      </c>
+      <c r="B26" t="s">
         <v>268</v>
       </c>
-      <c r="B26" t="s">
+      <c r="C26" t="s">
         <v>269</v>
-      </c>
-      <c r="C26" t="s">
-        <v>270</v>
       </c>
       <c r="E26" t="s">
         <v>48</v>
@@ -2497,7 +2542,7 @@
         <v>99</v>
       </c>
       <c r="Q26" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="S26" t="s">
         <v>156</v>
@@ -2511,13 +2556,13 @@
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B27" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C27" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E27" t="s">
         <v>49</v>
@@ -2525,13 +2570,13 @@
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
+        <v>274</v>
+      </c>
+      <c r="B28" t="s">
         <v>275</v>
       </c>
-      <c r="B28" t="s">
-        <v>276</v>
-      </c>
       <c r="C28" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E28" t="s">
         <v>50</v>
@@ -2539,13 +2584,13 @@
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B29" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C29" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E29" t="s">
         <v>51</v>
@@ -2556,13 +2601,13 @@
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B30" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C30" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E30" t="s">
         <v>52</v>
@@ -2571,35 +2616,35 @@
         <v>1</v>
       </c>
       <c r="N30" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
+        <v>283</v>
+      </c>
+      <c r="B31" t="s">
+        <v>283</v>
+      </c>
+      <c r="C31" t="s">
         <v>284</v>
-      </c>
-      <c r="B31" t="s">
-        <v>284</v>
-      </c>
-      <c r="C31" t="s">
-        <v>285</v>
       </c>
       <c r="E31" t="s">
         <v>53</v>
       </c>
       <c r="N31" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B32" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C32" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="E32" t="s">
         <v>54</v>
@@ -2608,35 +2653,35 @@
         <v>2</v>
       </c>
       <c r="N32" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
+        <v>293</v>
+      </c>
+      <c r="B33" t="s">
         <v>294</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
         <v>295</v>
-      </c>
-      <c r="C33" t="s">
-        <v>296</v>
       </c>
       <c r="E33" t="s">
         <v>55</v>
       </c>
       <c r="N33" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>298</v>
+      </c>
+      <c r="B34" t="s">
         <v>299</v>
       </c>
-      <c r="B34" t="s">
-        <v>300</v>
-      </c>
       <c r="C34" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E34" t="s">
         <v>56</v>
@@ -2645,35 +2690,35 @@
         <v>3</v>
       </c>
       <c r="N34" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
+        <v>301</v>
+      </c>
+      <c r="B35" t="s">
         <v>302</v>
       </c>
-      <c r="B35" t="s">
+      <c r="C35" t="s">
         <v>303</v>
       </c>
-      <c r="C35" t="s">
-        <v>304</v>
-      </c>
       <c r="E35" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="N35" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
+        <v>304</v>
+      </c>
+      <c r="B36" t="s">
         <v>305</v>
       </c>
-      <c r="B36" t="s">
-        <v>306</v>
-      </c>
       <c r="C36" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E36" t="s">
         <v>57</v>
@@ -2682,69 +2727,69 @@
         <v>4</v>
       </c>
       <c r="N36" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
+        <v>309</v>
+      </c>
+      <c r="B37" t="s">
         <v>310</v>
       </c>
-      <c r="B37" t="s">
-        <v>311</v>
-      </c>
       <c r="C37" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E37" t="s">
         <v>125</v>
       </c>
       <c r="N37" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B38" t="s">
+        <v>314</v>
+      </c>
+      <c r="C38" t="s">
         <v>315</v>
-      </c>
-      <c r="C38" t="s">
-        <v>316</v>
       </c>
       <c r="M38">
         <v>5</v>
       </c>
       <c r="N38" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
+        <v>317</v>
+      </c>
+      <c r="B39" t="s">
         <v>318</v>
       </c>
-      <c r="B39" t="s">
+      <c r="C39" t="s">
         <v>319</v>
-      </c>
-      <c r="C39" t="s">
-        <v>320</v>
       </c>
       <c r="E39" t="s">
         <v>58</v>
       </c>
       <c r="N39" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
+        <v>322</v>
+      </c>
+      <c r="B40" t="s">
         <v>323</v>
       </c>
-      <c r="B40" t="s">
+      <c r="C40" t="s">
         <v>324</v>
-      </c>
-      <c r="C40" t="s">
-        <v>325</v>
       </c>
       <c r="E40" t="s">
         <v>59</v>
@@ -2753,32 +2798,32 @@
         <v>6</v>
       </c>
       <c r="N40" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="B41" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C41" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="N41" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
+        <v>328</v>
+      </c>
+      <c r="B42" t="s">
         <v>329</v>
       </c>
-      <c r="B42" t="s">
-        <v>330</v>
-      </c>
       <c r="C42" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="E42" t="s">
         <v>60</v>
@@ -2787,24 +2832,24 @@
         <v>7</v>
       </c>
       <c r="N42" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
+        <v>340</v>
+      </c>
+      <c r="B43" t="s">
+        <v>346</v>
+      </c>
+      <c r="C43" t="s">
         <v>341</v>
-      </c>
-      <c r="B43" t="s">
-        <v>347</v>
-      </c>
-      <c r="C43" t="s">
-        <v>342</v>
       </c>
       <c r="E43" t="s">
         <v>61</v>
       </c>
       <c r="N43" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.3">
@@ -2826,30 +2871,30 @@
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="B45" t="s">
+        <v>348</v>
+      </c>
+      <c r="C45" t="s">
         <v>349</v>
-      </c>
-      <c r="C45" t="s">
-        <v>350</v>
       </c>
       <c r="E45" t="s">
         <v>62</v>
       </c>
       <c r="N45" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B46" t="s">
+        <v>350</v>
+      </c>
+      <c r="C46" t="s">
         <v>351</v>
-      </c>
-      <c r="C46" t="s">
-        <v>352</v>
       </c>
       <c r="E46" t="s">
         <v>63</v>
@@ -2860,22 +2905,31 @@
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
+        <v>343</v>
+      </c>
+      <c r="B47" t="s">
         <v>344</v>
       </c>
-      <c r="B47" t="s">
-        <v>345</v>
-      </c>
       <c r="C47" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="E47" t="s">
         <v>64</v>
       </c>
       <c r="N47" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>355</v>
+      </c>
+      <c r="B48" t="s">
+        <v>356</v>
+      </c>
+      <c r="C48" t="s">
+        <v>357</v>
+      </c>
       <c r="E48" t="s">
         <v>65</v>
       </c>
@@ -2883,15 +2937,33 @@
         <v>175</v>
       </c>
     </row>
-    <row r="49" spans="5:14" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>353</v>
+      </c>
+      <c r="B49" t="s">
+        <v>358</v>
+      </c>
+      <c r="C49" t="s">
+        <v>359</v>
+      </c>
       <c r="E49" t="s">
         <v>66</v>
       </c>
       <c r="N49" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="50" spans="5:14" x14ac:dyDescent="0.3">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>360</v>
+      </c>
+      <c r="B50" t="s">
+        <v>365</v>
+      </c>
+      <c r="C50" t="s">
+        <v>362</v>
+      </c>
       <c r="E50" t="s">
         <v>67</v>
       </c>
@@ -2899,12 +2971,30 @@
         <v>176</v>
       </c>
     </row>
-    <row r="51" spans="5:14" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>363</v>
+      </c>
+      <c r="B51" t="s">
+        <v>361</v>
+      </c>
+      <c r="C51" t="s">
+        <v>364</v>
+      </c>
       <c r="N51" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="52" spans="5:14" x14ac:dyDescent="0.3">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>366</v>
+      </c>
+      <c r="B52" t="s">
+        <v>368</v>
+      </c>
+      <c r="C52" t="s">
+        <v>367</v>
+      </c>
       <c r="E52" t="s">
         <v>88</v>
       </c>
@@ -2912,15 +3002,15 @@
         <v>177</v>
       </c>
     </row>
-    <row r="53" spans="5:14" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="E53" t="s">
         <v>68</v>
       </c>
       <c r="N53" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="54" spans="5:14" x14ac:dyDescent="0.3">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
       <c r="E54" t="s">
         <v>107</v>
       </c>
@@ -2928,14 +3018,14 @@
         <v>178</v>
       </c>
     </row>
-    <row r="55" spans="5:14" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="N55" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="56" spans="5:14" x14ac:dyDescent="0.3">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
       <c r="E56" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deployed 9ae3f80 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/Buch Bayrische Nächte/Sprache der Hölle.xlsx
+++ b/Buch Bayrische Nächte/Sprache der Hölle.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian Dauner\Documents\GitHub\pnpWiki\docs\Buch Bayrische Nächte\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5EC790C-5D06-4C8B-BC8D-E2D91631B918}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98EF9576-4517-4ACE-80ED-8CB473B18042}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="5205" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="369">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="391">
   <si>
     <t>Höllisch</t>
   </si>
@@ -813,9 +813,6 @@
     <t>command over</t>
   </si>
   <si>
-    <t>Shat-Tra-Ay</t>
-  </si>
-  <si>
     <t>Lustfull</t>
   </si>
   <si>
@@ -1065,9 +1062,6 @@
     <t>Food</t>
   </si>
   <si>
-    <t>Soulf of Body</t>
-  </si>
-  <si>
     <t>Feeder</t>
   </si>
   <si>
@@ -1132,6 +1126,78 @@
   </si>
   <si>
     <t>Body Ashbearer</t>
+  </si>
+  <si>
+    <t>Child</t>
+  </si>
+  <si>
+    <t>small Person</t>
+  </si>
+  <si>
+    <t>Mi-Rof</t>
+  </si>
+  <si>
+    <t>Sun</t>
+  </si>
+  <si>
+    <t>Fire Soul</t>
+  </si>
+  <si>
+    <t>Vra-Ru</t>
+  </si>
+  <si>
+    <t>Sunchild</t>
+  </si>
+  <si>
+    <t>deregatory for humans</t>
+  </si>
+  <si>
+    <t>Vra-Fu-Mi-Rof</t>
+  </si>
+  <si>
+    <t>to stop</t>
+  </si>
+  <si>
+    <t>Va-Lo-+Verb</t>
+  </si>
+  <si>
+    <t>Shat-Tra-+Verb</t>
+  </si>
+  <si>
+    <t>end Time</t>
+  </si>
+  <si>
+    <t>Soul of Body</t>
+  </si>
+  <si>
+    <t>Darkness</t>
+  </si>
+  <si>
+    <t>Nothing</t>
+  </si>
+  <si>
+    <t>Light</t>
+  </si>
+  <si>
+    <t>No Nothing</t>
+  </si>
+  <si>
+    <t>Va-Kor</t>
+  </si>
+  <si>
+    <t>Va-Va-Kor</t>
+  </si>
+  <si>
+    <t>God</t>
+  </si>
+  <si>
+    <t>godless</t>
+  </si>
+  <si>
+    <t>No God</t>
+  </si>
+  <si>
+    <t>Va-Nai</t>
   </si>
 </sst>
 </file>
@@ -1651,7 +1717,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W56"/>
+  <dimension ref="A1:W60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
@@ -1788,7 +1854,7 @@
         <v>186</v>
       </c>
       <c r="L3" s="4" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="M3" s="4" t="s">
         <v>223</v>
@@ -1946,13 +2012,13 @@
         <v>191</v>
       </c>
       <c r="R6" s="6" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="S6" s="6" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="T6" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="7" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2076,7 +2142,7 @@
         <v>194</v>
       </c>
       <c r="O9" s="6" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="P9" s="6" t="s">
         <v>249</v>
@@ -2182,7 +2248,7 @@
         <v>200</v>
       </c>
       <c r="J12" s="9" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="K12" s="9" t="s">
         <v>201</v>
@@ -2215,7 +2281,7 @@
         <v>69</v>
       </c>
       <c r="B14" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C14" t="s">
         <v>94</v>
@@ -2226,7 +2292,7 @@
         <v>122</v>
       </c>
       <c r="B15" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C15" t="s">
         <v>160</v>
@@ -2437,7 +2503,7 @@
         <v>259</v>
       </c>
       <c r="C23" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="N23" t="s">
         <v>100</v>
@@ -2466,7 +2532,7 @@
         <v>261</v>
       </c>
       <c r="C24" t="s">
-        <v>262</v>
+        <v>378</v>
       </c>
       <c r="E24" t="s">
         <v>46</v>
@@ -2478,7 +2544,7 @@
         <v>79</v>
       </c>
       <c r="Q24" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="S24" t="s">
         <v>161</v>
@@ -2492,13 +2558,13 @@
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B25" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C25" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="E25" t="s">
         <v>47</v>
@@ -2524,13 +2590,13 @@
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
+        <v>266</v>
+      </c>
+      <c r="B26" t="s">
         <v>267</v>
       </c>
-      <c r="B26" t="s">
+      <c r="C26" t="s">
         <v>268</v>
-      </c>
-      <c r="C26" t="s">
-        <v>269</v>
       </c>
       <c r="E26" t="s">
         <v>48</v>
@@ -2542,7 +2608,7 @@
         <v>99</v>
       </c>
       <c r="Q26" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="S26" t="s">
         <v>156</v>
@@ -2556,13 +2622,13 @@
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B27" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C27" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="E27" t="s">
         <v>49</v>
@@ -2570,13 +2636,13 @@
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
+        <v>273</v>
+      </c>
+      <c r="B28" t="s">
         <v>274</v>
       </c>
-      <c r="B28" t="s">
-        <v>275</v>
-      </c>
       <c r="C28" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="E28" t="s">
         <v>50</v>
@@ -2584,13 +2650,13 @@
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B29" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C29" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="E29" t="s">
         <v>51</v>
@@ -2601,13 +2667,13 @@
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B30" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C30" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="E30" t="s">
         <v>52</v>
@@ -2621,30 +2687,30 @@
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
+        <v>282</v>
+      </c>
+      <c r="B31" t="s">
+        <v>282</v>
+      </c>
+      <c r="C31" t="s">
         <v>283</v>
-      </c>
-      <c r="B31" t="s">
-        <v>283</v>
-      </c>
-      <c r="C31" t="s">
-        <v>284</v>
       </c>
       <c r="E31" t="s">
         <v>53</v>
       </c>
       <c r="N31" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B32" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C32" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="E32" t="s">
         <v>54</v>
@@ -2658,30 +2724,30 @@
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
+        <v>292</v>
+      </c>
+      <c r="B33" t="s">
         <v>293</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
         <v>294</v>
-      </c>
-      <c r="C33" t="s">
-        <v>295</v>
       </c>
       <c r="E33" t="s">
         <v>55</v>
       </c>
       <c r="N33" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>297</v>
+      </c>
+      <c r="B34" t="s">
         <v>298</v>
       </c>
-      <c r="B34" t="s">
-        <v>299</v>
-      </c>
       <c r="C34" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E34" t="s">
         <v>56</v>
@@ -2695,30 +2761,30 @@
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
+        <v>300</v>
+      </c>
+      <c r="B35" t="s">
         <v>301</v>
       </c>
-      <c r="B35" t="s">
+      <c r="C35" t="s">
         <v>302</v>
-      </c>
-      <c r="C35" t="s">
-        <v>303</v>
       </c>
       <c r="E35" t="s">
         <v>228</v>
       </c>
       <c r="N35" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
+        <v>303</v>
+      </c>
+      <c r="B36" t="s">
         <v>304</v>
       </c>
-      <c r="B36" t="s">
-        <v>305</v>
-      </c>
       <c r="C36" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E36" t="s">
         <v>57</v>
@@ -2732,30 +2798,30 @@
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
+        <v>308</v>
+      </c>
+      <c r="B37" t="s">
         <v>309</v>
       </c>
-      <c r="B37" t="s">
-        <v>310</v>
-      </c>
       <c r="C37" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E37" t="s">
         <v>125</v>
       </c>
       <c r="N37" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B38" t="s">
+        <v>313</v>
+      </c>
+      <c r="C38" t="s">
         <v>314</v>
-      </c>
-      <c r="C38" t="s">
-        <v>315</v>
       </c>
       <c r="M38">
         <v>5</v>
@@ -2766,30 +2832,30 @@
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
+        <v>316</v>
+      </c>
+      <c r="B39" t="s">
         <v>317</v>
       </c>
-      <c r="B39" t="s">
+      <c r="C39" t="s">
         <v>318</v>
-      </c>
-      <c r="C39" t="s">
-        <v>319</v>
       </c>
       <c r="E39" t="s">
         <v>58</v>
       </c>
       <c r="N39" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
+        <v>321</v>
+      </c>
+      <c r="B40" t="s">
         <v>322</v>
       </c>
-      <c r="B40" t="s">
+      <c r="C40" t="s">
         <v>323</v>
-      </c>
-      <c r="C40" t="s">
-        <v>324</v>
       </c>
       <c r="E40" t="s">
         <v>59</v>
@@ -2803,27 +2869,27 @@
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B41" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C41" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="N41" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
+        <v>327</v>
+      </c>
+      <c r="B42" t="s">
         <v>328</v>
       </c>
-      <c r="B42" t="s">
-        <v>329</v>
-      </c>
       <c r="C42" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E42" t="s">
         <v>60</v>
@@ -2832,24 +2898,24 @@
         <v>7</v>
       </c>
       <c r="N42" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
+        <v>339</v>
+      </c>
+      <c r="B43" t="s">
+        <v>380</v>
+      </c>
+      <c r="C43" t="s">
         <v>340</v>
-      </c>
-      <c r="B43" t="s">
-        <v>346</v>
-      </c>
-      <c r="C43" t="s">
-        <v>341</v>
       </c>
       <c r="E43" t="s">
         <v>61</v>
       </c>
       <c r="N43" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.3">
@@ -2871,30 +2937,30 @@
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B45" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C45" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="E45" t="s">
         <v>62</v>
       </c>
       <c r="N45" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="B46" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="C46" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="E46" t="s">
         <v>63</v>
@@ -2905,30 +2971,30 @@
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
+        <v>342</v>
+      </c>
+      <c r="B47" t="s">
         <v>343</v>
       </c>
-      <c r="B47" t="s">
-        <v>344</v>
-      </c>
       <c r="C47" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="E47" t="s">
         <v>64</v>
       </c>
       <c r="N47" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
+        <v>353</v>
+      </c>
+      <c r="B48" t="s">
+        <v>354</v>
+      </c>
+      <c r="C48" t="s">
         <v>355</v>
-      </c>
-      <c r="B48" t="s">
-        <v>356</v>
-      </c>
-      <c r="C48" t="s">
-        <v>357</v>
       </c>
       <c r="E48" t="s">
         <v>65</v>
@@ -2939,30 +3005,30 @@
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="B49" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="C49" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="E49" t="s">
         <v>66</v>
       </c>
       <c r="N49" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
+        <v>358</v>
+      </c>
+      <c r="B50" t="s">
+        <v>363</v>
+      </c>
+      <c r="C50" t="s">
         <v>360</v>
-      </c>
-      <c r="B50" t="s">
-        <v>365</v>
-      </c>
-      <c r="C50" t="s">
-        <v>362</v>
       </c>
       <c r="E50" t="s">
         <v>67</v>
@@ -2973,27 +3039,27 @@
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="B51" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C51" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="N51" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
+        <v>364</v>
+      </c>
+      <c r="B52" t="s">
         <v>366</v>
       </c>
-      <c r="B52" t="s">
-        <v>368</v>
-      </c>
       <c r="C52" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="E52" t="s">
         <v>88</v>
@@ -3003,14 +3069,32 @@
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>367</v>
+      </c>
+      <c r="B53" t="s">
+        <v>368</v>
+      </c>
+      <c r="C53" t="s">
+        <v>369</v>
+      </c>
       <c r="E53" t="s">
         <v>68</v>
       </c>
       <c r="N53" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>370</v>
+      </c>
+      <c r="B54" t="s">
+        <v>371</v>
+      </c>
+      <c r="C54" t="s">
+        <v>372</v>
+      </c>
       <c r="E54" t="s">
         <v>107</v>
       </c>
@@ -3019,13 +3103,75 @@
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>373</v>
+      </c>
+      <c r="B55" t="s">
+        <v>374</v>
+      </c>
+      <c r="C55" t="s">
+        <v>375</v>
+      </c>
       <c r="N55" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>376</v>
+      </c>
+      <c r="B56" t="s">
+        <v>379</v>
+      </c>
+      <c r="C56" t="s">
+        <v>377</v>
+      </c>
       <c r="E56" t="s">
-        <v>342</v>
+        <v>341</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>381</v>
+      </c>
+      <c r="B57" t="s">
+        <v>382</v>
+      </c>
+      <c r="C57" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>383</v>
+      </c>
+      <c r="B58" t="s">
+        <v>384</v>
+      </c>
+      <c r="C58" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>387</v>
+      </c>
+      <c r="B59" t="s">
+        <v>387</v>
+      </c>
+      <c r="C59" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>388</v>
+      </c>
+      <c r="B60" t="s">
+        <v>389</v>
+      </c>
+      <c r="C60" t="s">
+        <v>390</v>
       </c>
     </row>
   </sheetData>

</xml_diff>